<commit_message>
feat: update master dictionary and keyword cache for Hungary and Spain, adding new demographic options and correcting variable names
</commit_message>
<xml_diff>
--- a/data/country_maps/hungary_review.xlsx
+++ b/data/country_maps/hungary_review.xlsx
@@ -748,76 +748,76 @@
       <c r="L6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>born1</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Mikor születtél? – Év</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>When were you born? – Year | 2000 | 2001 | 2002 | 2003 | 2004 | 2005 | 2006 | 2007 | 2008 | 2009 | 2010 | 2011</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>byear1</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>What year were you born?</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>2000 | 2001 | 2002 | 2003 | 2004 | 2005 | 2006 | 2007 | 2008 | 2009 | 2010 | 2011</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>schooltype</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Melyik felsőoktatási intézménybe, és milyen szakra jársz? - Selected Choice</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Which higher education institution and what major do you attend? - Selected Choice</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>grade1</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>What grade are you in?</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>8th | 9th | 10th | 11th | 12th | 13th | Graduated from school | Quit school before graduating</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Manual fix: B-export grade equivalent</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>sleep4</t>
+          <t>born4_1_TEXT</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MENTOR kérdőív</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Mióta vannak éjszakai megébredéseid?</t>
+          <t>Körülbelül hány éves voltál, amikor Magyarországra jöttél/költöztél? - Kor: - Text</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Kevesebb mint 1 hónapja | 1-2 hónapja | 3-6 hónapja | 7-11 hónapja | 1-3 éve | Több mint 3 éve | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>How long have you had nighttime awakenings? | Less than 1 month | 1-2 months | 3-6 months | 7-11 months | 1-3 years | More than 3 years | Prefer not to answer | Don't know / Not applicable</t>
+          <t>Approximately how old were you when you came/moved to Hungary? - Age: - Text</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -834,28 +834,24 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>sleep5</t>
+          <t>ethnic1_7_TEXT</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>MENTOR kérdőív</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran vagy fáradt vagy álmos napközben?</t>
+          <t>Melyik etnikai közösséghez tartozol?  Kérjük, jelöld be az összes rád illőt! Több választ is megjelölhetsz! - Egyéb: - Text</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Soha | Néhányszor | Heti 1 nap | Heti 2-3 nap | Heti 4-5 nap | Heti 6-7 nap | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
-        </is>
-      </c>
+      <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>How often are you tired or sleepy during the day? | Never | A few times | 1 day a week | 2-3 days a week | 4-5 days a week | 6-7 days a week | Prefer not to answer | Don't know / Not applicable</t>
+          <t>Which ethnic community do you belong to? Please select all that apply! You may select multiple answers! - Other: - Text</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -870,47 +866,55 @@
       <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>sleep6</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>MENTOR kérdőív</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Mióta érzed magad fáradtnak vagy álmosnak napközben?</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Kevesebb mint 1 hónapja | 1-2 hónapja | 3-6 hónapja | 7-11 hónapja | 1-3 éve | Több mint 3 éve | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>How long have you felt tired or sleepy during the day? | Less than 1 month | 1-2 months | 3-6 months | 7-11 months | 1-3 years | More than 3 years | Prefer not to answer | Don't know / Not applicable</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>born1</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Mikor születtél? – Év</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>When were you born? – Year | 2000 | 2001 | 2002 | 2003 | 2004 | 2005 | 2006 | 2007 | 2008 | 2009 | 2010 | 2011</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>byear1</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>What year were you born?</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>2000 | 2001 | 2002 | 2003 | 2004 | 2005 | 2006 | 2007 | 2008 | 2009 | 2010 | 2011</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>sleep7</t>
+          <t>sleep4</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -920,18 +924,18 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hétköznapokon általában mikor fekszel le aludni?</t>
+          <t>Mióta vannak éjszakai megébredéseid?</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>20:00 előtt | 20:00 és 20:29 között | 20:30 és 20:59 között | 21:00 és 21:29 között | 21:30 és 21:59 között | 22:00 és 22:29 között | 22:30 és 22:59 között | 23:00 és 23:29 között | 23:30 és 23:59 között | 00:00 és 00:29 között | 00:30 és 00:59 között | 01:00 és 01:29 között | 01:30 és 01:59 között | 02:00 és 02:29 között | 02:30 és 02:59 között | 03:00 után | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+          <t>Kevesebb mint 1 hónapja | 1-2 hónapja | 3-6 hónapja | 7-11 hónapja | 1-3 éve | Több mint 3 éve | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>On weekdays, what time do you usually go to bed to sleep? | Before 20:00 | Between 20:00 and 20:29 | Between 20:30 and 20:59 | Between 21:00 and 21:29 | Between 21:30 and 21:59 | Between 22:00 and 22:29 | Between 22:30 and 22:59 | Between 23:00 and 23:29 | Between 23:30 and 23:59 | Between 00:00 and 00:29 | Between 00:30 and 00:59 | Between 01:00 and 01:29 | Between 01:30 and 01:59 | Between 02:00 and 02:29 | Between 02:30 and 02:59 | After 03:00 | Prefer not to answer | Don't know / Not applicable</t>
+          <t>How long have you had nighttime awakenings? | Less than 1 month | 1-2 months | 3-6 months | 7-11 months | 1-3 years | More than 3 years | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -948,7 +952,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>sleep8</t>
+          <t>sleep5</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -958,18 +962,18 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétköznap mennyi időbe telik elaludnod miután lefekszel?</t>
+          <t>Milyen gyakran vagy fáradt vagy álmos napközben?</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Kevesebb, mint 30 perc | 30 perc és 1 óra között | 1 és 1,5 óra között | 1,5 és 2 óra között | Több, mint 2 óra | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+          <t>Soha | Néhányszor | Heti 1 nap | Heti 2-3 nap | Heti 4-5 nap | Heti 6-7 nap | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>On an average weekday, how long does it take you to fall asleep after going to bed? | Less than 30 minutes | Between 30 minutes and 1 hour | Between 1 and 1.5 hours | Between 1.5 and 2 hours | More than 2 hours | Prefer not to answer | Don't know / Not applicable</t>
+          <t>How often are you tired or sleepy during the day? | Never | A few times | 1 day a week | 2-3 days a week | 4-5 days a week | 6-7 days a week | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -986,7 +990,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>sleep9</t>
+          <t>sleep6</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -996,18 +1000,18 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hétköznapokon mennyi ideig vagy ébren éjszaka (az első elalvás után)?</t>
+          <t>Mióta érzed magad fáradtnak vagy álmosnak napközben?</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Kevesebb, mint 30 perc | 30 perc és 1 óra között | 1 és 1,5 óra között | 1,5 és 2 óra között | Több, mint 2 óra | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+          <t>Kevesebb mint 1 hónapja | 1-2 hónapja | 3-6 hónapja | 7-11 hónapja | 1-3 éve | Több mint 3 éve | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>On weekdays, how long are you awake at night (after first falling asleep)? | Less than 30 minutes | Between 30 minutes and 1 hour | Between 1 and 1.5 hours | Between 1.5 and 2 hours | More than 2 hours | Prefer not to answer | Don't know / Not applicable</t>
+          <t>How long have you felt tired or sleepy during the day? | Less than 1 month | 1-2 months | 3-6 months | 7-11 months | 1-3 years | More than 3 years | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1024,7 +1028,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>sleep10</t>
+          <t>sleep7</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1034,18 +1038,18 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hétköznap általában mikor ébredsz reggelente?</t>
+          <t>Hétköznapokon általában mikor fekszel le aludni?</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>05:00 előtt | 05:00 és 05:29 között | 05:30 és 05:59 között | 06:00 és 06:29 között | 06:30 és 06:59 között | 07:00 és 07:29 között | 07:30 és 07:59 között | 08:00 és 08:29 között | 08:30 és 08:59 között | 09:00 és 09:29 között | 09:30 és 09:59 között | 10:00 után | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+          <t>20:00 előtt | 20:00 és 20:29 között | 20:30 és 20:59 között | 21:00 és 21:29 között | 21:30 és 21:59 között | 22:00 és 22:29 között | 22:30 és 22:59 között | 23:00 és 23:29 között | 23:30 és 23:59 között | 00:00 és 00:29 között | 00:30 és 00:59 között | 01:00 és 01:29 között | 01:30 és 01:59 között | 02:00 és 02:29 között | 02:30 és 02:59 között | 03:00 után | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>On weekdays, what time do you usually wake up in the morning? | Before 05:00 | Between 05:00 and 05:29 | Between 05:30 and 05:59 | Between 06:00 and 06:29 | Between 06:30 and 06:59 | Between 07:00 and 07:29 | Between 07:30 and 07:59 | Between 08:00 and 08:29 | Between 08:30 and 08:59 | Between 09:00 and 09:29 | Between 09:30 and 09:59 | After 10:00 | Prefer not to answer | Don't know / Not applicable to me</t>
+          <t>On weekdays, what time do you usually go to bed to sleep? | Before 20:00 | Between 20:00 and 20:29 | Between 20:30 and 20:59 | Between 21:00 and 21:29 | Between 21:30 and 21:59 | Between 22:00 and 22:29 | Between 22:30 and 22:59 | Between 23:00 and 23:29 | Between 23:30 and 23:59 | Between 00:00 and 00:29 | Between 00:30 and 00:59 | Between 01:00 and 01:29 | Between 01:30 and 01:59 | Between 02:00 and 02:29 | Between 02:30 and 02:59 | After 03:00 | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
@@ -1062,7 +1066,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>sleep11</t>
+          <t>sleep8</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1072,18 +1076,18 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használsz elektronikus eszközöket (pl. mobiltelefon, tablet, PC/Mac, TV stb.) a hálószobádban a lefekvés előtti utolsó órában?</t>
+          <t>Egy átlagos hétköznap mennyi időbe telik elaludnod miután lefekszel?</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Soha/ritkán | Heti 1-2 este | Heti 3-6 este | Minden este | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+          <t>Kevesebb, mint 30 perc | 30 perc és 1 óra között | 1 és 1,5 óra között | 1,5 és 2 óra között | Több, mint 2 óra | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>How often do you use electronic devices (e.g., mobile phone, tablet, PC/Mac, TV, etc.) in your bedroom during the last hour before going to sleep? | Never/rarely | 1-2 nights a week | 3-6 nights a week | Every night | Prefer not to answer | Don't know / Not applicable to me</t>
+          <t>On an average weekday, how long does it take you to fall asleep after going to bed? | Less than 30 minutes | Between 30 minutes and 1 hour | Between 1 and 1.5 hours | Between 1.5 and 2 hours | More than 2 hours | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
@@ -1100,7 +1104,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>sleep12</t>
+          <t>sleep9</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1110,18 +1114,18 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran küldesz vagy fogadsz üzeneteket este, lefekvés után?</t>
+          <t>Hétköznapokon mennyi ideig vagy ébren éjszaka (az első elalvás után)?</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Soha/ritkán | Heti 1-2 este | Heti 3-6 este | Minden este | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Szülőkkel való kapcsolat</t>
+          <t>Kevesebb, mint 30 perc | 30 perc és 1 óra között | 1 és 1,5 óra között | 1,5 és 2 óra között | Több, mint 2 óra | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>How often do you send or receive messages in the evening after going to bed? | Never/rarely | 1-2 nights a week | 3-6 nights a week | Every night | Prefer not to answer | Don't know / Not applicable to me | Relationship with parents</t>
+          <t>On weekdays, how long are you awake at night (after first falling asleep)? | Less than 30 minutes | Between 30 minutes and 1 hour | Between 1 and 1.5 hours | Between 1.5 and 2 hours | More than 2 hours | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
@@ -1138,7 +1142,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>repa1:8_1</t>
+          <t>sleep10</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1148,18 +1152,18 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban.</t>
+          <t>Hétköznap általában mikor ébredsz reggelente?</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Soha | Néha | Gyakran | Szinte mindig | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | A szüleim megértenek engem | Jól kijövök a szüleimmel | A szüleim kedvelnek engem | Kedvelem a szüleimet | A szüleim kritizálnak | A szüleim idegesítenek | A szüleim megbántanak engem | Vitatkozunk a szüleimmel | Kapcsolat a barátokkal</t>
+          <t>05:00 előtt | 05:00 és 05:29 között | 05:30 és 05:59 között | 06:00 és 06:29 között | 06:30 és 06:59 között | 07:00 és 07:29 között | 07:30 és 07:59 között | 08:00 és 08:29 között | 08:30 és 08:59 között | 09:00 és 09:29 között | 09:30 és 09:59 között | 10:00 után | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. | Never | Sometimes | Often | Almost always | Prefer not to answer | Don't know / Not applicable to me | My parents understand me | I get along well with my parents | My parents like me | I like my parents | My parents criticize me | My parents annoy me | My parents hurt me | We argue with my parents | Relationship with friends</t>
+          <t>On weekdays, what time do you usually wake up in the morning? | Before 05:00 | Between 05:00 and 05:29 | Between 05:30 and 05:59 | Between 06:00 and 06:29 | Between 06:30 and 06:59 | Between 07:00 and 07:29 | Between 07:30 and 07:59 | Between 08:00 and 08:29 | Between 08:30 and 08:59 | Between 09:00 and 09:29 | Between 09:30 and 09:59 | After 10:00 | Prefer not to answer | Don't know / Not applicable to me</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
@@ -1176,7 +1180,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>refr1:5_1</t>
+          <t>sleep11</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1186,18 +1190,18 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Mennyire érvényesek rád az alábbi állítások?</t>
+          <t>Milyen gyakran használsz elektronikus eszközöket (pl. mobiltelefon, tablet, PC/Mac, TV stb.) a hálószobádban a lefekvés előtti utolsó órában?</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Egyáltalán nem értek egyet | Nem értek egyet | Egyetértek | Teljes mértékben egyetértek | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Elég nehéznek találom a barátkozást | Sok barátom van | A többi fiatal nehéznek találja, hogy kedveljen engem | Népszerű vagyok a többi fiatal körében | Érzem, hogy mások elfogadnak</t>
+          <t>Soha/ritkán | Heti 1-2 este | Heti 3-6 este | Minden este | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>To what extent do the following statements apply to you? | Strongly disagree | Disagree | Agree | Strongly agree | Prefer not to answer | Don't know / Not applicable to me | I find it quite difficult to make friends | I have a lot of friends | Other young people find it hard to like me | I am popular among other young people | I feel accepted by others</t>
+          <t>How often do you use electronic devices (e.g., mobile phone, tablet, PC/Mac, TV, etc.) in your bedroom during the last hour before going to sleep? | Never/rarely | 1-2 nights a week | 3-6 nights a week | Every night | Prefer not to answer | Don't know / Not applicable to me</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
@@ -1214,7 +1218,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>relationship1</t>
+          <t>sleep12</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1224,18 +1228,18 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Van barátod vagy barátnőd, jársz valakivel?</t>
+          <t>Milyen gyakran küldesz vagy fogadsz üzeneteket este, lefekvés után?</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Van | Nincs, de korábban már volt | Nincs, és még nem is volt | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Szabadidő</t>
+          <t>Soha/ritkán | Heti 1-2 este | Heti 3-6 este | Minden este | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Szülőkkel való kapcsolat</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Do you have a boyfriend or girlfriend, are you dating someone? | Yes | No, but have had before | No, and have never had | Prefer not to answer | Don't know / Not applicable to me | Leisure time</t>
+          <t>How often do you send or receive messages in the evening after going to bed? | Never/rarely | 1-2 nights a week | 3-6 nights a week | Every night | Prefer not to answer | Don't know / Not applicable to me | Relationship with parents</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
@@ -1252,7 +1256,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>leisure1:5_1</t>
+          <t>repa1:8_1</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1262,18 +1266,18 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket?</t>
+          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Soha/ritkán | 1 nap | 2-3 nap | 4-5 nap | 6-7 nap | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Időt tölteni a barátaiddal | Edzeni (pl. foci, kézilabda, síelés, futás, tánc, torna) | Részt venni más szervezett tevékenységekben (pl. színház, zene, cserkészkedés) | Egész délután és este otthon maradni | Könyveket olvasni vagy hangoskönyveket hallgatni | Az iskolán kívül: Hetente körülbelül hány órát sportolsz úgy vagy végzel olyan fizikai tevékenységet (pl. foci, kézilabda, futás, torna, tánc stb.), amelyben kifulladsz vagy izzadsz? Amennyiben nem tudod vagy nem szeretnél válaszolni, kérjük, írd be az alábbi cellába, hogy "Nem tudom" vagy "Nem szeretnék válaszolni"!</t>
+          <t>Soha | Néha | Gyakran | Szinte mindig | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | A szüleim megértenek engem | Jól kijövök a szüleimmel | A szüleim kedvelnek engem | Kedvelem a szüleimet | A szüleim kritizálnak | A szüleim idegesítenek | A szüleim megbántanak engem | Vitatkozunk a szüleimmel | Kapcsolat a barátokkal</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Outside of school: On how many days in an average week do you usually do the following? | Never/rarely | 1 day | 2-3 days | 4-5 days | 6-7 days | Prefer not to answer | Don't know / Not applicable to me | Spend time with your friends | Exercise (e.g., football, handball, skiing, running, dancing, gymnastics) | Participate in other organized activities (e.g., theater, music, scouting) | Stay at home all afternoon and evening | Read books or listen to audiobooks | Outside of school: Approximately how many hours per week do you play sports or do physical activity (e.g., football, handball, running, gymnastics, dancing, etc.) that makes you breathe hard or sweat? If you do not know or do not wish to answer, please enter "Don't know" or "Prefer not to answer" in the cell below!</t>
+          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. | Never | Sometimes | Often | Almost always | Prefer not to answer | Don't know / Not applicable to me | My parents understand me | I get along well with my parents | My parents like me | I like my parents | My parents criticize me | My parents annoy me | My parents hurt me | We argue with my parents | Relationship with friends</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
@@ -1290,7 +1294,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>activity_week1:5_1</t>
+          <t>refr1:5_1</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1300,18 +1304,18 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel?</t>
+          <t>Mennyire érvényesek rád az alábbi állítások?</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Soha/ritkán | Kevesebb mint 1 órát | 1-2 órát | 3-4 órát | 5-6 órát | 7 vagy több órát | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Film/sorozat/TV nézés | Házi feladat elkészítése | Játék PC-n (asztali számítógépen), TV-n, tableten, telefonon stb. | Leülni a számítógép elé, vagy leülni/lefeküdni telefonnal vagy táblagéppel (tevékenységtől függetlenül) | A közösségi media aktív használata (nem csak bejelentkezve lenni)</t>
+          <t>Egyáltalán nem értek egyet | Nem értek egyet | Egyetértek | Teljes mértékben egyetértek | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Elég nehéznek találom a barátkozást | Sok barátom van | A többi fiatal nehéznek találja, hogy kedveljen engem | Népszerű vagyok a többi fiatal körében | Érzem, hogy mások elfogadnak</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>On an average weekday, how much time do you spend on the following activities? | Never/rarely | Less than 1 hour | 1-2 hours | 3-4 hours | 5-6 hours | 7 or more hours | Prefer not to answer | Don't know / Not applicable to me | Watching movies/series/TV | Doing homework | Gaming on PC (desktop computer), TV, tablet, phone, etc. | Sitting in front of the computer, or sitting/lying down with a phone or tablet (regardless of activity) | Actively using social media (not just being logged in)</t>
+          <t>To what extent do the following statements apply to you? | Strongly disagree | Disagree | Agree | Strongly agree | Prefer not to answer | Don't know / Not applicable to me | I find it quite difficult to make friends | I have a lot of friends | Other young people find it hard to like me | I am popular among other young people | I feel accepted by others</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
@@ -1328,7 +1332,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>activity_weekend1:5_1</t>
+          <t>relationship1</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1338,18 +1342,18 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel?</t>
+          <t>Van barátod vagy barátnőd, jársz valakivel?</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Soha/ritkán | Kevesebb mint 1 órát | 1-2 órát | 3-4 órát | 5-6 órát | 7 vagy több órát | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Film/sorozat/TV nézés | Házi feladat elkészítése | Játék PC-n (asztali számítógépen), TV-n, tableten, telefonon stb. | Leülni a számítógép elé, vagy leülni/lefeküdni telefonnal vagy táblagéppel (tevékenységtől függetlenül) | A közösségi media aktív használata (nem csak bejelentkezve lenni)</t>
+          <t>Van | Nincs, de korábban már volt | Nincs, és még nem is volt | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Szabadidő</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>On an average weekend day or holiday, how much time do you spend on the following activities? | Never/rarely | Less than 1 hour | 1-2 hours | 3-4 hours | 5-6 hours | 7 or more hours | Prefer not to answer | Don't know / Not applicable to me | Watching movies/series/TV | Doing homework | Gaming on PC (desktop computer), TV, tablet, phone, etc. | Sitting in front of the computer, or sitting/lying down with a phone or tablet (regardless of activity) | Actively using social media (not just being logged in)</t>
+          <t>Do you have a boyfriend or girlfriend, are you dating someone? | Yes | No, but have had before | No, and have never had | Prefer not to answer | Don't know / Not applicable to me | Leisure time</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
@@ -1366,7 +1370,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>training1</t>
+          <t>leisure1:5_1</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1376,18 +1380,18 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Részt veszel szervezett edzéseken (sportklubokon vagy szervezeteken keresztül)?</t>
+          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket?</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Igen | Nem, de korábban részt vettem | Nem | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Hány évesen hagytad abba a szervezett sportolást? Amennyiben nem tudod vagy nem szeretnél válaszolni, kérjük, írd be az alábbi cellába, hogy "Nem tudom" vagy "Nem szeretnék válaszolni"! | Kiegészítő kérdések | 10 | Iskola</t>
+          <t>Soha/ritkán | 1 nap | 2-3 nap | 4-5 nap | 6-7 nap | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Időt tölteni a barátaiddal | Edzeni (pl. foci, kézilabda, síelés, futás, tánc, torna) | Részt venni más szervezett tevékenységekben (pl. színház, zene, cserkészkedés) | Egész délután és este otthon maradni | Könyveket olvasni vagy hangoskönyveket hallgatni | Az iskolán kívül: Hetente körülbelül hány órát sportolsz úgy vagy végzel olyan fizikai tevékenységet (pl. foci, kézilabda, futás, torna, tánc stb.), amelyben kifulladsz vagy izzadsz? Amennyiben nem tudod vagy nem szeretnél válaszolni, kérjük, írd be az alábbi cellába, hogy "Nem tudom" vagy "Nem szeretnék válaszolni"!</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Do you participate in organized training (through sports clubs or organizations)? | Yes | No, but participated before | No | Prefer not to answer | Don't know / Not applicable to me | At what age did you stop participating in organized sports? If you do not know or do not wish to answer, please enter "Don't know" or "Prefer not to answer" in the cell below! | Supplementary questions | 10 | School</t>
+          <t>Outside of school: On how many days in an average week do you usually do the following? | Never/rarely | 1 day | 2-3 days | 4-5 days | 6-7 days | Prefer not to answer | Don't know / Not applicable to me | Spend time with your friends | Exercise (e.g., football, handball, skiing, running, dancing, gymnastics) | Participate in other organized activities (e.g., theater, music, scouting) | Stay at home all afternoon and evening | Read books or listen to audiobooks | Outside of school: Approximately how many hours per week do you play sports or do physical activity (e.g., football, handball, running, gymnastics, dancing, etc.) that makes you breathe hard or sweat? If you do not know or do not wish to answer, please enter "Don't know" or "Prefer not to answer" in the cell below!</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
@@ -1404,7 +1408,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>school1:11_1</t>
+          <t>activity_week1:5_1</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1414,18 +1418,18 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal!</t>
+          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel?</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Teljesen mértékben egyetértek | Inkább egyetértek | Inkább nem értek egyet | Egyáltalán nem értek egyet | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Élvezem az iskolát. | A tanáraim törődnek velem. | Úgy érzem, beilleszkedem a diákok közé az iskolában. | Unatkozom az iskolában. | Sokan azt várják tőlem, hogy jól teljesítsek az iskolában. | Gyakran rettegek iskolába menni. | A hétvégéket gyakran iskolai munkával kell töltenem. | Túl sok a zaj és a rendbontás az órákon. | Az iskolában sok az elvesztegetett idő. | Sok érdekes dolgot tanulunk az iskolában. | Fontos a jó jegyek megszerzése.</t>
+          <t>Soha/ritkán | Kevesebb mint 1 órát | 1-2 órát | 3-4 órát | 5-6 órát | 7 vagy több órát | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Film/sorozat/TV nézés | Házi feladat elkészítése | Játék PC-n (asztali számítógépen), TV-n, tableten, telefonon stb. | Leülni a számítógép elé, vagy leülni/lefeküdni telefonnal vagy táblagéppel (tevékenységtől függetlenül) | A közösségi media aktív használata (nem csak bejelentkezve lenni)</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! | Strongly agree | Somewhat agree | Somewhat disagree | Strongly disagree | Prefer not to answer | Don't know / Not applicable to me | I enjoy school. | My teachers care about me. | I feel like I fit in among the students at school. | I am bored at school. | Many people expect me to perform well at school. | I often dread going to school. | I often have to spend weekends doing schoolwork. | There is too much noise and disruption in classes. | A lot of time is wasted at school. | We learn many interesting things at school. | Getting good grades is important.</t>
+          <t>On an average weekday, how much time do you spend on the following activities? | Never/rarely | Less than 1 hour | 1-2 hours | 3-4 hours | 5-6 hours | 7 or more hours | Prefer not to answer | Don't know / Not applicable to me | Watching movies/series/TV | Doing homework | Gaming on PC (desktop computer), TV, tablet, phone, etc. | Sitting in front of the computer, or sitting/lying down with a phone or tablet (regardless of activity) | Actively using social media (not just being logged in)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -1442,7 +1446,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>school_stress1:3_1</t>
+          <t>activity_weekend1:5_1</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1452,18 +1456,18 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Iskolai stressz</t>
+          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel?</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Soha | Ritkán | Néha | Gyakran | Nagyon gyakran | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Stresszes leszek az iskolai feladatoktól | Kimerültnek érzem magam az iskolai feladatok miatt. | Több iskolai feladatom van, mint amennyit kezelni tudok. | Köszönjük, hogy kitöltötted a kérdőívet! | Amennyiben úgy érzed, hogy a kérdőívben feltett kérdések felkavaróak voltak a számodra, ezért azok rád gyakorolt hatását szeretnéd megbeszélni valakivel, kérjük, hogy keresd őket az alábbi elérhetőségeken: Kék Vonal Gyermekkrízis Alapítvány 116-111 (éjjel-nappal hívható, ingyenes) Magyar Lelki Elsősegély Telefonszolgálatok Szövetsége (LESZ) 116-123 (éjjel-nappal hívható, ingyenes)</t>
+          <t>Soha/ritkán | Kevesebb mint 1 órát | 1-2 órát | 3-4 órát | 5-6 órát | 7 vagy több órát | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Film/sorozat/TV nézés | Házi feladat elkészítése | Játék PC-n (asztali számítógépen), TV-n, tableten, telefonon stb. | Leülni a számítógép elé, vagy leülni/lefeküdni telefonnal vagy táblagéppel (tevékenységtől függetlenül) | A közösségi media aktív használata (nem csak bejelentkezve lenni)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>School stress | Never | Rarely | Sometimes | Often | Very often | Prefer not to answer | Don't know / Not applicable to me | I get stressed from schoolwork | I feel exhausted because of schoolwork. | I have more schoolwork than I can handle. | Thank you for completing the questionnaire! | If you feel that the questions in the survey were upsetting to you and you would like to discuss their impact on you with someone, please contact them at the following: Kék Vonal Child Crisis Foundation 116-111 (toll-free, available 24/7) Hungarian Mental First Aid Telephone Services Association (LESZ) 116-123 (toll-free, available 24/7)</t>
+          <t>On an average weekend day or holiday, how much time do you spend on the following activities? | Never/rarely | Less than 1 hour | 1-2 hours | 3-4 hours | 5-6 hours | 7 or more hours | Prefer not to answer | Don't know / Not applicable to me | Watching movies/series/TV | Doing homework | Gaming on PC (desktop computer), TV, tablet, phone, etc. | Sitting in front of the computer, or sitting/lying down with a phone or tablet (regardless of activity) | Actively using social media (not just being logged in)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
@@ -1478,319 +1482,319 @@
       <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>training1</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>MENTOR kérdőív</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Részt veszel szervezett edzéseken (sportklubokon vagy szervezeteken keresztül)?</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Igen | Nem, de korábban részt vettem | Nem | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Hány évesen hagytad abba a szervezett sportolást? Amennyiben nem tudod vagy nem szeretnél válaszolni, kérjük, írd be az alábbi cellába, hogy "Nem tudom" vagy "Nem szeretnék válaszolni"! | Kiegészítő kérdések | 10 | Iskola</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Do you participate in organized training (through sports clubs or organizations)? | Yes | No, but participated before | No | Prefer not to answer | Don't know / Not applicable to me | At what age did you stop participating in organized sports? If you do not know or do not wish to answer, please enter "Don't know" or "Prefer not to answer" in the cell below! | Supplementary questions | 10 | School</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>school1:11_1</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>MENTOR kérdőív</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal!</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Teljesen mértékben egyetértek | Inkább egyetértek | Inkább nem értek egyet | Egyáltalán nem értek egyet | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Élvezem az iskolát. | A tanáraim törődnek velem. | Úgy érzem, beilleszkedem a diákok közé az iskolában. | Unatkozom az iskolában. | Sokan azt várják tőlem, hogy jól teljesítsek az iskolában. | Gyakran rettegek iskolába menni. | A hétvégéket gyakran iskolai munkával kell töltenem. | Túl sok a zaj és a rendbontás az órákon. | Az iskolában sok az elvesztegetett idő. | Sok érdekes dolgot tanulunk az iskolában. | Fontos a jó jegyek megszerzése.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Please indicate how much you agree with the following statements! | Strongly agree | Somewhat agree | Somewhat disagree | Strongly disagree | Prefer not to answer | Don't know / Not applicable to me | I enjoy school. | My teachers care about me. | I feel like I fit in among the students at school. | I am bored at school. | Many people expect me to perform well at school. | I often dread going to school. | I often have to spend weekends doing schoolwork. | There is too much noise and disruption in classes. | A lot of time is wasted at school. | We learn many interesting things at school. | Getting good grades is important.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>school_stress1:3_1</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>MENTOR kérdőív</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Iskolai stressz</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Soha | Ritkán | Néha | Gyakran | Nagyon gyakran | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Stresszes leszek az iskolai feladatoktól | Kimerültnek érzem magam az iskolai feladatok miatt. | Több iskolai feladatom van, mint amennyit kezelni tudok. | Köszönjük, hogy kitöltötted a kérdőívet! | Amennyiben úgy érzed, hogy a kérdőívben feltett kérdések felkavaróak voltak a számodra, ezért azok rád gyakorolt hatását szeretnéd megbeszélni valakivel, kérjük, hogy keresd őket az alábbi elérhetőségeken: Kék Vonal Gyermekkrízis Alapítvány 116-111 (éjjel-nappal hívható, ingyenes) Magyar Lelki Elsősegély Telefonszolgálatok Szövetsége (LESZ) 116-123 (éjjel-nappal hívható, ingyenes)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>School stress | Never | Rarely | Sometimes | Often | Very often | Prefer not to answer | Don't know / Not applicable to me | I get stressed from schoolwork | I feel exhausted because of schoolwork. | I have more schoolwork than I can handle. | Thank you for completing the questionnaire! | If you feel that the questions in the survey were upsetting to you and you would like to discuss their impact on you with someone, please contact them at the following: Kék Vonal Child Crisis Foundation 116-111 (toll-free, available 24/7) Hungarian Mental First Aid Telephone Services Association (LESZ) 116-123 (toll-free, available 24/7)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>born2</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Mikor születtél? – Hónap</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>When were you born? – Month | January | February | March | April | May | June | July | August | September | October | November | December</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>bmonth1</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>What month were you born?</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr"/>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>January | February | March | April | May | June | July | August | September | October | November | December</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>matched</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>born3</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>MENTOR kérdőív</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Hol születtél?</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr"/>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Magyarország | Albánia | Andorra | Ausztria | Belgium | Bosznia-Hercegovina | Bulgária | Csehország | Dánia | Egyesült Királyság | Észak-Macedónia | Észtország | Fehéroro­szország | Finnország | Franciaország | Görögország | Hollandia | Horvátország | Írország | Izland | Lengyelország | Lettország | Liechtenstein | Litvánia | Luxemburg | Málta | Moldova | Monaco | Montenegró | Németország | Norvégia | Olaszország | Oroszország | Portugália | Románia | San Marino | Spanyolország | Svájc | Svédország | Szerbia | Szlovákia | Szlovénia | Törökország | Ukrajna | Vatikán | Egyéb európai terület | Közel-Kelet vagy Észak-Afrika | Szubszaharai Afrika | Ázsia | Észak-Amerika | Dél- vagy Közép-Amerika | Egyéb | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Körülbelül hány éves voltál, amikor Magyarországra jöttél/költöztél? Amennyiben nem tudod vagy nem szeretnél válaszolni, kérjük, írd be az alábbi cellába, hogy "Nem tudom" vagy "Nem szeretnék válaszolni"!</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>Where were you born? | Hungary | Albania | Andorra | Austria | Belgium | Bosnia and Herzegovina | Bulgaria | Czech Republic | Denmark | United Kingdom | North Macedonia | Estonia | Belarus | Finland | France | Greece | Netherlands | Croatia | Ireland | Iceland | Poland | Latvia | Liechtenstein | Lithuania | Luxembourg | Malta | Moldova | Monaco | Montenegro | Germany | Norway | Italy | Russia | Portugal | Romania | San Marino | Spain | Switzerland | Sweden | Serbia | Slovakia | Slovenia | Turkey | Ukraine | Vatican | Other European territory | Middle East or North Africa | Sub-Saharan Africa | Asia | North America | South or Central America | Other | Prefer not to answer | Don't know / Not applicable to me | Approximately how old were you when you came/moved to Hungary? If you do not know or do not wish to answer, please type "Don't know" or "Prefer not to answer" in the box below!</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>bplace1</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>Where were you born?</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="5" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>[COUNTRY] | Ukraine | Albania | Andorra | Austria | Belarus | Belgium | Bosnia and Herzegovina | Bulgaria | Croatia | Cyprus | Czech Republic | Denmark | Estonia | Finland | France | Germany | Greece | Hungary | Iceland | Ireland | Italy | Kosovo | Latvia | Liechtenstein | Lithuania | Luxembourg | Malta | Moldova | Monaco | Montenegro | Netherlands | North Macedonia | Norway | Poland | Portugal | Romania | Russia | Serbia | Slovakia | Slovenia | Spain | Sweden | Switzerland | Turkey | United Kingdom | Middle East or North Africa | Sub-Saharan Africa | Asia | North America | South or Central America | Oseania | Other</t>
         </is>
       </c>
-      <c r="K27" s="5" t="inlineStr">
+      <c r="K30" s="5" t="inlineStr">
         <is>
           <t>probable</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="L30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>sleep3</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>MENTOR kérdőív</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Milyen gyakran történik meg, hogy felébredsz éjszakánként?</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr"/>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Soha | Néhányszor | Heti 1 nap | Heti 2-3 nap | Heti 4-5 nap | Heti 6-7 nap | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>How often do you wake up during the night? | Never | A few times | 1 day a week | 2-3 days a week | 4-5 days a week | 6-7 days a week | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>bage1</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Approximately how old were you when you came/moved to [country]?</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr"/>
-      <c r="J28" s="6" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr"/>
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>0 | 1 | 2 | 3 | 4 | 5 | 6 | 7 | 8 | 9 | 10 | 11 | 12 | 13 | 14 | 15 | 16 | 17 | 18</t>
         </is>
       </c>
-      <c r="K28" s="6" t="inlineStr">
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>conflict</t>
         </is>
       </c>
-      <c r="L28" s="6" t="inlineStr">
+      <c r="L31" s="6" t="inlineStr">
         <is>
           <t>Fallback text match (0.41)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>born4</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Körülbelül hány éves voltál, amikor Magyarországra jöttél/költöztél? - Selected Choice</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr"/>
-      <c r="E29" s="6" t="inlineStr"/>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Approximately how old were you when you came/moved to Hungary? - Selected Choice | 0 | 1 | 2 | 3 | 4 | 5 | 6 | 7 | 8 | 9 | 10 | 11 | 12 | 13 | 14 | 15 | 16 | 17 | 18</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>bage1</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Approximately how old were you when you came/moved to [country]?</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr"/>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr"/>
+      <c r="J32" s="6" t="inlineStr">
         <is>
           <t>0 | 1 | 2 | 3 | 4 | 5 | 6 | 7 | 8 | 9 | 10 | 11 | 12 | 13 | 14 | 15 | 16 | 17 | 18</t>
         </is>
       </c>
-      <c r="K29" s="6" t="inlineStr">
+      <c r="K32" s="6" t="inlineStr">
         <is>
           <t>conflict</t>
         </is>
       </c>
-      <c r="L29" s="6" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>dasc01:25_1</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>MENTOR kérdőív</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb. Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok!</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Soha | Ritkán | Néha | Gyakran | Mindig | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Amikor nem vagyok iskolában, sok időt töltök az eszközöm használatával | Azt érzem, hogy több időt kell töltenem az eszközöm használatával | Feszült leszek, ha nem tudom használni az eszközömet | Hazudok a szüleimnek arról, hogy mennyi időt töltök az eszközöm használatával | Az eszközöm használata segít elfelejteni a problémáimat | Nem töltök időt a családtagjaimmal, mert szívesebben használom az eszközömet | Egyre több időt töltök az eszközöm használatával | Ideges leszek, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát | A szüleim megpróbálják megakadályozni vagy korlátozni az eszközöm használatát, de nem sikerül nekik | Kevesebbet alszom az eszközöm használata miatt | Amikor nincs nálam az eszközöm, arra gondolok, amit azon szoktam csinálni (videojátékok, közösségi média, üzenetek stb.) | Feszült vagyok, ha nem tudom használni az eszközömet. | Konfliktusaim vannak a szüleimmel azzal kapcsolatban, hogy mennyi időt töltök az eszközöm használatával | Az eszközöm használata a legfontosabb dolog az életemben | Az eszközöm használata élvezetesebb, mint más dolgok | Hazudok a szüleimnek arról, hogy mit csinálok az eszközömön | Nem tudom uralni az eszközöm használatát | Elvesztettem érdeklődésemet hobbik vagy más tevékenységek iránt, mert inkább az eszközömet használom | Amikor abbahagyom az eszközöm használatát, nem sokkal később újra elkezdem használni | Megnézem az eszközöm, amikor házi feladatot vagy más fontos dolgot csinálok | Feszült leszek, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát | Összeveszek a szüleimmel, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát | Túl sok pénzt költök az eszközömhöz kapcsolódó dolgokra | Amikor rosszkedvű vagyok, az eszközöm használatától jobb kedvem lesz | Továbbra is használom az eszközöm annak ellenére, hogy az iskolai jegyeim egyre rosszabbak | C-SSRS és szerhasználat | 8 | Columbia súlyosságértékelő skála öngyilkosság kockázatára (C-SSRS)</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>When you read the word "device" in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. "Using my device" means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you during the past week. There are no right or wrong answers! | Never | Rarely | Sometimes | Often | Always | Prefer not to answer | Don't know / Not applicable | When I am not at school, I spend a lot of time using my device | I feel that I need to spend more time using my device | I get tense if I cannot use my device | I lie to my parents about how much time I spend using my device | Using my device helps me forget my problems | I do not spend time with family members because I prefer to use my device | I spend more and more time using my device | I get annoyed when I am asked to stop using my device | My parents try to prevent or limit my device use, but they fail | I sleep less because of using my device | When I don't have my device with me, I think about what I usually do on it (video games, social media, messages, etc.) | I am tense if I cannot use my device. | I have conflicts with my parents about how much time I spend using my device | Using my device is the most important thing in my life | Using my device is more enjoyable than other things | I lie to my parents about what I do on my device | I cannot control my device use | I have lost interest in hobbies or other activities because I prefer using my device | When I stop using my device, not long after I start using it again | I check my device when doing homework or other important things | I get tense when I am asked to stop using my device | I argue with my parents when I am asked to stop using my device | I spend too much money on things related to my device | When I am in a bad mood, using my device makes me feel better | I continue to use my device even though my school grades are getting worse | C-SSRS and substance use | 8 | Columbia-Suicide Severity Rating Scale (C-SSRS)</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>suicide1:5_1</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>MENTOR kérdőív</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha?</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Igen, a múltban - egyszer | Igen, a múltban - többször | Igen, az elmúlt 30 napban | Igen, a múltban és az elmúlt 30 napban is | Nem, soha | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Kívántad már, hogy meghalj, vagy hogy elaludj, és ne ébredj fel? | Voltak ténylegesen olyan gondolataid, hogy megölöd magad? | Gondolkodtál már azon, hogy hogyan ölhetnéd meg magad? | Elkezdtél-e kidolgozni, esetleg ténylegesen ki is dolgoztál részleteket, hogy hogyan öld meg magad, és szándékodban is állt megvalósítani ezt a tervet? | Kíséreltél már meg öngyilkosságot? | Amennyiben kíséreltél már meg öngyilkosságot, hány alkalommal? Amennyiben nem tudod vagy nem szeretnél válaszolni, kérjük, írd be az alábbi cellába, hogy "Nem tudom" vagy "Nem szeretnék válaszolni"! | Szerhasználat | Milyen gyakran használtad az alábbi dohánytermékeket az elmúlt 30 nap során ? | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Cigaretta | E-cigaretta (pl. iqos, elfbar, poco) | Szájba helyezett dohány (snus) | Milyen gyakran használtad az alábbi dohánytermékeket az életed során ? | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Cigaretta | E-cigaretta (pl. iqos, elfbar, poco) | Szájba helyezett dohány (snus) | Kérjük, jelöld a válaszokat az alábbiak alapján: | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Milyen gyakran fogyasztottál alkoholos italokat (pl. sör, alkoholos üdítőital, bor, rövid italok/shotok) az elmúlt 30 nap során ?</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? | Yes, in the past - once | Yes, in the past - several times | Yes, in the past 30 days | Yes, both in the past and in the past 30 days | No, never | Prefer not to answer | Don't know / Not applicable | Have you wished you were dead or wished you could go to sleep and not wake up? | Have you actually had thoughts of killing yourself? | Have you been thinking about how you might kill yourself? | Have you started to work out or actually worked out the details of how to kill yourself, and did you have some intention to carry out this plan? | Have you ever attempted suicide? | If you have ever attempted suicide, how many times? If you don't know or do not wish to answer, please type "Don't know" or "Prefer not to answer" into the cell below! | Substance use | How often have you used the following tobacco products during the past 30 days? | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | Cigarettes | E-cigarettes (e.g. IQOS, Elf Bar, Poco) | Oral tobacco (snus) | How often have you used the following tobacco products during your lifetime? | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | Cigarettes | E-cigarettes (e.g. IQOS, Elf Bar, Poco) | Oral tobacco (snus) | Please mark your answers based on the following: | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | How often did you consume alcoholic beverages (e.g. beer, alcopops/cider, wine, spirits/shots) during the past 30 days?</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>sub_abuse8</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>MENTOR kérdőív</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Milyen gyakran ittál életed során bármilyen alkoholt?</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Milyen gyakran rúgtál be az elmúlt 30 nap során ? | Milyen gyakran rugtál be életed során ?</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>How often have you drunk any alcohol during your lifetime? | How often did you get drunk during the past 30 days? | How often did you get drunk during your lifetime?</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse11</t>
+          <t>dasc01:25_1</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1800,18 +1804,18 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Ha valaha volt ilyen, milyen gyakran ittál meg 5 vagy több alkoholos italt (pl. sör, alkoholos üdítőital, bor, rövid italok/shotok) egy óra vagy annál kevesebb idő alatt? Milyen gyakran használtál életed során olyan vényköteles gyógyszert, amelyet nem neked írtak fel (pl. nyugtatók, stimulánsok)? Milyen gyakran használtál életed során olyan tudatmódosító szert, amelyet nem tekintenek kábítószernek (például ragasztót, gázt, festéket vagy patront)? Használtál valaha valamilyen drogot?</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb. Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok!</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Igen | Nem | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során ? | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Kábítószer cigarettában elszívva | Kábítószer szájon át bevéve | Kábítószer orrba felszippantva | Kábítószer intravénásan (érbe) befecskendezve | Milyen gyakran használtad az alábbi kábítószereket életed során ? | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Kábítószer cigarettában elszívva | Kábítószer szájon át bevéve | Kábítószer orrba felszippantva | Kábítószer intravénásan (érbe) befecskendezve | Alvás, kapcsolatok és szabadidő | 9 | Alvás</t>
+          <t>Soha | Ritkán | Néha | Gyakran | Mindig | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Amikor nem vagyok iskolában, sok időt töltök az eszközöm használatával | Azt érzem, hogy több időt kell töltenem az eszközöm használatával | Feszült leszek, ha nem tudom használni az eszközömet | Hazudok a szüleimnek arról, hogy mennyi időt töltök az eszközöm használatával | Az eszközöm használata segít elfelejteni a problémáimat | Nem töltök időt a családtagjaimmal, mert szívesebben használom az eszközömet | Egyre több időt töltök az eszközöm használatával | Ideges leszek, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát | A szüleim megpróbálják megakadályozni vagy korlátozni az eszközöm használatát, de nem sikerül nekik | Kevesebbet alszom az eszközöm használata miatt | Amikor nincs nálam az eszközöm, arra gondolok, amit azon szoktam csinálni (videojátékok, közösségi média, üzenetek stb.) | Feszült vagyok, ha nem tudom használni az eszközömet. | Konfliktusaim vannak a szüleimmel azzal kapcsolatban, hogy mennyi időt töltök az eszközöm használatával | Az eszközöm használata a legfontosabb dolog az életemben | Az eszközöm használata élvezetesebb, mint más dolgok | Hazudok a szüleimnek arról, hogy mit csinálok az eszközömön | Nem tudom uralni az eszközöm használatát | Elvesztettem érdeklődésemet hobbik vagy más tevékenységek iránt, mert inkább az eszközömet használom | Amikor abbahagyom az eszközöm használatát, nem sokkal később újra elkezdem használni | Megnézem az eszközöm, amikor házi feladatot vagy más fontos dolgot csinálok | Feszült leszek, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát | Összeveszek a szüleimmel, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát | Túl sok pénzt költök az eszközömhöz kapcsolódó dolgokra | Amikor rosszkedvű vagyok, az eszközöm használatától jobb kedvem lesz | Továbbra is használom az eszközöm annak ellenére, hogy az iskolai jegyeim egyre rosszabbak | C-SSRS és szerhasználat | 8 | Columbia súlyosságértékelő skála öngyilkosság kockázatára (C-SSRS)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>If ever, how often did you drink 5 or more alcoholic drinks (e.g. beer, alcopops/cider, wine, spirits/shots) in an hour or less? How often in your lifetime have you used prescription medication that was not prescribed to you (e.g. sedatives, stimulants)? How often in your lifetime have you used mind-altering substances that are not considered drugs (such as glue, gas, paint, or whippets)? Have you ever used any drugs? | Yes | No | Prefer not to answer | Don't know / Not applicable | How often have you used the following drugs during the past 30 days? | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | Drugs smoked in a cigarette | Drugs taken orally | Drugs snorted through the nose | Drugs injected intravenously (into a vein) | How often have you used the following drugs during your lifetime? | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | Drugs smoked in a cigarette | Drugs taken orally | Drugs snorted through the nose | Drugs injected intravenously (into a vein) | Sleep, relationships and leisure | 9 | Sleep</t>
+          <t>When you read the word "device" in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. "Using my device" means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you during the past week. There are no right or wrong answers! | Never | Rarely | Sometimes | Often | Always | Prefer not to answer | Don't know / Not applicable | When I am not at school, I spend a lot of time using my device | I feel that I need to spend more time using my device | I get tense if I cannot use my device | I lie to my parents about how much time I spend using my device | Using my device helps me forget my problems | I do not spend time with family members because I prefer to use my device | I spend more and more time using my device | I get annoyed when I am asked to stop using my device | My parents try to prevent or limit my device use, but they fail | I sleep less because of using my device | When I don't have my device with me, I think about what I usually do on it (video games, social media, messages, etc.) | I am tense if I cannot use my device. | I have conflicts with my parents about how much time I spend using my device | Using my device is the most important thing in my life | Using my device is more enjoyable than other things | I lie to my parents about what I do on my device | I cannot control my device use | I have lost interest in hobbies or other activities because I prefer using my device | When I stop using my device, not long after I start using it again | I check my device when doing homework or other important things | I get tense when I am asked to stop using my device | I argue with my parents when I am asked to stop using my device | I spend too much money on things related to my device | When I am in a bad mood, using my device makes me feel better | I continue to use my device even though my school grades are getting worse | C-SSRS and substance use | 8 | Columbia-Suicide Severity Rating Scale (C-SSRS)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
@@ -1828,7 +1832,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>sleep1</t>
+          <t>suicide1:5_1</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1838,18 +1842,18 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran okoz számodra nehézséget az éjszakai elalvás?</t>
+          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha?</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Soha | Néhányszor | Heti 1 nap | Heti 2-3 nap | Heti 4-5 nap | Heti 6-7 nap | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+          <t>Igen, a múltban - egyszer | Igen, a múltban - többször | Igen, az elmúlt 30 napban | Igen, a múltban és az elmúlt 30 napban is | Nem, soha | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Kívántad már, hogy meghalj, vagy hogy elaludj, és ne ébredj fel? | Voltak ténylegesen olyan gondolataid, hogy megölöd magad? | Gondolkodtál már azon, hogy hogyan ölhetnéd meg magad? | Elkezdtél-e kidolgozni, esetleg ténylegesen ki is dolgoztál részleteket, hogy hogyan öld meg magad, és szándékodban is állt megvalósítani ezt a tervet? | Kíséreltél már meg öngyilkosságot? | Amennyiben kíséreltél már meg öngyilkosságot, hány alkalommal? Amennyiben nem tudod vagy nem szeretnél válaszolni, kérjük, írd be az alábbi cellába, hogy "Nem tudom" vagy "Nem szeretnék válaszolni"! | Szerhasználat | Milyen gyakran használtad az alábbi dohánytermékeket az elmúlt 30 nap során ? | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Cigaretta | E-cigaretta (pl. iqos, elfbar, poco) | Szájba helyezett dohány (snus) | Milyen gyakran használtad az alábbi dohánytermékeket az életed során ? | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Cigaretta | E-cigaretta (pl. iqos, elfbar, poco) | Szájba helyezett dohány (snus) | Kérjük, jelöld a válaszokat az alábbiak alapján: | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Milyen gyakran fogyasztottál alkoholos italokat (pl. sör, alkoholos üdítőital, bor, rövid italok/shotok) az elmúlt 30 nap során ?</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>How often do you have difficulty falling asleep at night? | Never | A few times | 1 day a week | 2-3 days a week | 4-5 days a week | 6-7 days a week | Prefer not to answer | Don't know / Not applicable</t>
+          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? | Yes, in the past - once | Yes, in the past - several times | Yes, in the past 30 days | Yes, both in the past and in the past 30 days | No, never | Prefer not to answer | Don't know / Not applicable | Have you wished you were dead or wished you could go to sleep and not wake up? | Have you actually had thoughts of killing yourself? | Have you been thinking about how you might kill yourself? | Have you started to work out or actually worked out the details of how to kill yourself, and did you have some intention to carry out this plan? | Have you ever attempted suicide? | If you have ever attempted suicide, how many times? If you don't know or do not wish to answer, please type "Don't know" or "Prefer not to answer" into the cell below! | Substance use | How often have you used the following tobacco products during the past 30 days? | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | Cigarettes | E-cigarettes (e.g. IQOS, Elf Bar, Poco) | Oral tobacco (snus) | How often have you used the following tobacco products during your lifetime? | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | Cigarettes | E-cigarettes (e.g. IQOS, Elf Bar, Poco) | Oral tobacco (snus) | Please mark your answers based on the following: | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | How often did you consume alcoholic beverages (e.g. beer, alcopops/cider, wine, spirits/shots) during the past 30 days?</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
@@ -1866,7 +1870,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>sleep2</t>
+          <t>sub_abuse8</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1876,18 +1880,18 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Mióta okoz számodra nehézséget az éjszakai elalvás?</t>
+          <t>Milyen gyakran ittál életed során bármilyen alkoholt?</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Kevesebb mint 1 hónapja | 1-2 hónapja | 3-6 hónapja | 7-11 hónapja | 1-3 éve | Több mint 3 éve | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+          <t>Milyen gyakran rúgtál be az elmúlt 30 nap során ? | Milyen gyakran rugtál be életed során ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>How long have you been having difficulty falling asleep at night? | Less than 1 month | 1-2 months | 3-6 months | 7-11 months | 1-3 years | More than 3 years | Prefer not to answer | Don't know / Not applicable</t>
+          <t>How often have you drunk any alcohol during your lifetime? | How often did you get drunk during the past 30 days? | How often did you get drunk during your lifetime?</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
@@ -1904,24 +1908,28 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>born4_1_TEXT</t>
+          <t>sub_abuse11</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>MENTOR kérdőív</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Körülbelül hány éves voltál, amikor Magyarországra jöttél/költöztél? - Kor: - Text</t>
+          <t>Ha valaha volt ilyen, milyen gyakran ittál meg 5 vagy több alkoholos italt (pl. sör, alkoholos üdítőital, bor, rövid italok/shotok) egy óra vagy annál kevesebb idő alatt? Milyen gyakran használtál életed során olyan vényköteles gyógyszert, amelyet nem neked írtak fel (pl. nyugtatók, stimulánsok)? Milyen gyakran használtál életed során olyan tudatmódosító szert, amelyet nem tekintenek kábítószernek (például ragasztót, gázt, festéket vagy patront)? Használtál valaha valamilyen drogot?</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Igen | Nem | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során ? | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Kábítószer cigarettában elszívva | Kábítószer szájon át bevéve | Kábítószer orrba felszippantva | Kábítószer intravénásan (érbe) befecskendezve | Milyen gyakran használtad az alábbi kábítószereket életed során ? | Soha | 1-2-szer | 3-5-ször | 6-9-szer | 10-19-szer | 20-39-szer | 40-szer vagy többször | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Kábítószer cigarettában elszívva | Kábítószer szájon át bevéve | Kábítószer orrba felszippantva | Kábítószer intravénásan (érbe) befecskendezve | Alvás, kapcsolatok és szabadidő | 9 | Alvás</t>
+        </is>
+      </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Approximately how old were you when you came/moved to Hungary? - Age: - Text</t>
+          <t>If ever, how often did you drink 5 or more alcoholic drinks (e.g. beer, alcopops/cider, wine, spirits/shots) in an hour or less? How often in your lifetime have you used prescription medication that was not prescribed to you (e.g. sedatives, stimulants)? How often in your lifetime have you used mind-altering substances that are not considered drugs (such as glue, gas, paint, or whippets)? Have you ever used any drugs? | Yes | No | Prefer not to answer | Don't know / Not applicable | How often have you used the following drugs during the past 30 days? | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | Drugs smoked in a cigarette | Drugs taken orally | Drugs snorted through the nose | Drugs injected intravenously (into a vein) | How often have you used the following drugs during your lifetime? | Never | 1-2 times | 3-5 times | 6-9 times | 10-19 times | 20-39 times | 40 or more times | Prefer not to answer | Don't know / Not applicable | Drugs smoked in a cigarette | Drugs taken orally | Drugs snorted through the nose | Drugs injected intravenously (into a vein) | Sleep, relationships and leisure | 9 | Sleep</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
@@ -1938,24 +1946,28 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>schooltype</t>
+          <t>sleep1</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>MENTOR kérdőív</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Melyik felsőoktatási intézménybe, és milyen szakra jársz? - Selected Choice</t>
+          <t>Milyen gyakran okoz számodra nehézséget az éjszakai elalvás?</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Soha | Néhányszor | Heti 1 nap | Heti 2-3 nap | Heti 4-5 nap | Heti 6-7 nap | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+        </is>
+      </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Which higher education institution and what major do you attend? - Selected Choice</t>
+          <t>How often do you have difficulty falling asleep at night? | Never | A few times | 1 day a week | 2-3 days a week | 4-5 days a week | 6-7 days a week | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
@@ -1972,24 +1984,28 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ethnic1_7_TEXT</t>
+          <t>sleep2</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>MENTOR kérdőív</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Melyik etnikai közösséghez tartozol?  Kérjük, jelöld be az összes rád illőt! Több választ is megjelölhetsz! - Egyéb: - Text</t>
+          <t>Mióta okoz számodra nehézséget az éjszakai elalvás?</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Kevesebb mint 1 hónapja | 1-2 hónapja | 3-6 hónapja | 7-11 hónapja | 1-3 éve | Több mint 3 éve | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám</t>
+        </is>
+      </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Which ethnic community do you belong to? Please select all that apply! You may select multiple answers! - Other: - Text</t>
+          <t>How long have you been having difficulty falling asleep at night? | Less than 1 month | 1-2 months | 3-6 months | 7-11 months | 1-3 years | More than 3 years | Prefer not to answer | Don't know / Not applicable</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -8880,47 +8896,67 @@
       <c r="L170" s="5" t="inlineStr"/>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="inlineStr">
+      <c r="A171" s="3" t="inlineStr">
         <is>
           <t>some_use1:6_1</t>
         </is>
       </c>
-      <c r="B171" s="2" t="inlineStr">
+      <c r="B171" s="3" t="inlineStr">
         <is>
           <t>MENTOR kérdőív</t>
         </is>
       </c>
-      <c r="C171" s="2" t="inlineStr">
+      <c r="C171" s="3" t="inlineStr">
         <is>
           <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata!</t>
         </is>
       </c>
-      <c r="D171" s="2" t="inlineStr"/>
-      <c r="E171" s="2" t="inlineStr">
+      <c r="D171" s="3" t="inlineStr"/>
+      <c r="E171" s="3" t="inlineStr">
         <is>
           <t>Szinte mindig | Gyakran | Néha | Ritkán | Soha | Nem szeretnék válaszolni | Nem tudom / Nem vonatkozik rám | Alvás | Iskolai feladatok | Önbecsülés/mentális egészség | Baráti kapcsolatok | Családi kapcsolatok | Szabadtéri tevékenységek vagy sportolás</t>
         </is>
       </c>
-      <c r="F171" s="2" t="inlineStr">
+      <c r="F171" s="3" t="inlineStr">
         <is>
           <t>Please indicate for the following areas of life how often the use of phone, computer, or game console has a negative impact on them! | Almost always | Often | Sometimes | Rarely | Never | Prefer not to answer | Don't know / Not applicable | Sleep | School assignments | Self-esteem/mental health | Friendships | Family relationships | Outdoor activities or sports</t>
         </is>
       </c>
-      <c r="G171" s="2" t="inlineStr"/>
-      <c r="H171" s="2" t="inlineStr"/>
-      <c r="I171" s="2" t="inlineStr"/>
-      <c r="J171" s="2" t="inlineStr"/>
-      <c r="K171" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L171" s="2" t="inlineStr"/>
+      <c r="G171" s="3" t="inlineStr">
+        <is>
+          <t>smharm1</t>
+        </is>
+      </c>
+      <c r="H171" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="inlineStr">
+        <is>
+          <t>Sleep</t>
+        </is>
+      </c>
+      <c r="J171" s="3" t="inlineStr">
+        <is>
+          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="K171" s="3" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="L171" s="3" t="inlineStr">
+        <is>
+          <t>Manual fix: first smharm item (was unmapped)</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>dasc01:25_10</t>
+          <t>some_use1:6_2</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -8930,19 +8966,19 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Kevesebbet alszom az eszközöm használata miatt</t>
+          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Iskolai feladatok</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr"/>
       <c r="E172" s="3" t="inlineStr"/>
       <c r="F172" s="3" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I sleep less because of using my device</t>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Schoolwork | Nearly all the time | Often | Sometimes | Rarely | Never</t>
         </is>
       </c>
       <c r="G172" s="3" t="inlineStr">
         <is>
-          <t>smharm1</t>
+          <t>smharm2</t>
         </is>
       </c>
       <c r="H172" s="3" t="inlineStr">
@@ -8952,7 +8988,7 @@
       </c>
       <c r="I172" s="3" t="inlineStr">
         <is>
-          <t>Sleep</t>
+          <t>Schoolwork</t>
         </is>
       </c>
       <c r="J172" s="3" t="inlineStr">
@@ -8965,152 +9001,212 @@
           <t>matched</t>
         </is>
       </c>
-      <c r="L172" s="3" t="inlineStr">
-        <is>
-          <t>Fallback text match (1.00)</t>
-        </is>
-      </c>
+      <c r="L172" s="3" t="inlineStr"/>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="inlineStr">
-        <is>
-          <t>some_apps1_15_TEXT</t>
-        </is>
-      </c>
-      <c r="B173" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C173" s="2" t="inlineStr">
-        <is>
-          <t>Kérjük, jelöld be azt a három alkalmazást vagy szolgáltatást, amelyeket a leggyakrabban használod! - Egyéb: - Text</t>
-        </is>
-      </c>
-      <c r="D173" s="2" t="inlineStr"/>
-      <c r="E173" s="2" t="inlineStr"/>
-      <c r="F173" s="2" t="inlineStr">
-        <is>
-          <t>Please select the three apps or services that you use most often! - Other: - Text</t>
-        </is>
-      </c>
-      <c r="G173" s="2" t="inlineStr"/>
-      <c r="H173" s="2" t="inlineStr"/>
-      <c r="I173" s="2" t="inlineStr"/>
-      <c r="J173" s="2" t="inlineStr"/>
-      <c r="K173" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L173" s="2" t="inlineStr"/>
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>some_use1:6_3</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Önbecsülés/mentális egészség</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr"/>
+      <c r="E173" s="3" t="inlineStr"/>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Self-esteem/mental health | Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="G173" s="3" t="inlineStr">
+        <is>
+          <t>smharm3</t>
+        </is>
+      </c>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="inlineStr">
+        <is>
+          <t>Self-esteem/mental health</t>
+        </is>
+      </c>
+      <c r="J173" s="3" t="inlineStr">
+        <is>
+          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="K173" s="3" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="L173" s="3" t="inlineStr"/>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>dasc01:25_2</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C174" s="2" t="inlineStr">
-        <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Azt érzem, hogy több időt kell töltenem az eszközöm használatával</t>
-        </is>
-      </c>
-      <c r="D174" s="2" t="inlineStr"/>
-      <c r="E174" s="2" t="inlineStr"/>
-      <c r="F174" s="2" t="inlineStr">
-        <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Select the answer that was true for you during the past week. There are no right or wrong answers! - I feel that I need to spend more time using my device</t>
-        </is>
-      </c>
-      <c r="G174" s="2" t="inlineStr"/>
-      <c r="H174" s="2" t="inlineStr"/>
-      <c r="I174" s="2" t="inlineStr"/>
-      <c r="J174" s="2" t="inlineStr"/>
-      <c r="K174" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L174" s="2" t="inlineStr"/>
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>some_use1:6_4</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Baráti kapcsolatok</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr"/>
+      <c r="E174" s="3" t="inlineStr"/>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Friendships / relationships with friends | Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="G174" s="3" t="inlineStr">
+        <is>
+          <t>smharm4</t>
+        </is>
+      </c>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
+          <t>Relationships with friends</t>
+        </is>
+      </c>
+      <c r="J174" s="3" t="inlineStr">
+        <is>
+          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="K174" s="3" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="L174" s="3" t="inlineStr"/>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="inlineStr">
-        <is>
-          <t>dasc01:25_3</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C175" s="2" t="inlineStr">
-        <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Feszült leszek, ha nem tudom használni az eszközömet</t>
-        </is>
-      </c>
-      <c r="D175" s="2" t="inlineStr"/>
-      <c r="E175" s="2" t="inlineStr"/>
-      <c r="F175" s="2" t="inlineStr">
-        <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Select the answer that was true for you during the past week. There are no right or wrong answers! - I become tense if I cannot use my device</t>
-        </is>
-      </c>
-      <c r="G175" s="2" t="inlineStr"/>
-      <c r="H175" s="2" t="inlineStr"/>
-      <c r="I175" s="2" t="inlineStr"/>
-      <c r="J175" s="2" t="inlineStr"/>
-      <c r="K175" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L175" s="2" t="inlineStr"/>
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>some_use1:6_5</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Családi kapcsolatok</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr"/>
+      <c r="E175" s="3" t="inlineStr"/>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Family relationships / relationships with family | Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="G175" s="3" t="inlineStr">
+        <is>
+          <t>smharm5</t>
+        </is>
+      </c>
+      <c r="H175" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="inlineStr">
+        <is>
+          <t>Relationships with family</t>
+        </is>
+      </c>
+      <c r="J175" s="3" t="inlineStr">
+        <is>
+          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="K175" s="3" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="L175" s="3" t="inlineStr"/>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>dasc01:25_4</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C176" s="2" t="inlineStr">
-        <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Hazudok a szüleimnek arról, hogy mennyi időt töltök az eszközöm használatával</t>
-        </is>
-      </c>
-      <c r="D176" s="2" t="inlineStr"/>
-      <c r="E176" s="2" t="inlineStr"/>
-      <c r="F176" s="2" t="inlineStr">
-        <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Select the answer that was true for you during the past week. There are no right or wrong answers! - I lie to my parents about how much time I spend using my device</t>
-        </is>
-      </c>
-      <c r="G176" s="2" t="inlineStr"/>
-      <c r="H176" s="2" t="inlineStr"/>
-      <c r="I176" s="2" t="inlineStr"/>
-      <c r="J176" s="2" t="inlineStr"/>
-      <c r="K176" s="2" t="inlineStr">
-        <is>
-          <t>extra</t>
-        </is>
-      </c>
-      <c r="L176" s="2" t="inlineStr"/>
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>some_use1:6_6</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Szabadtéri tevékenységek vagy sportolás</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr"/>
+      <c r="E176" s="3" t="inlineStr"/>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Outdoor activities or sports | Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="G176" s="3" t="inlineStr">
+        <is>
+          <t>smharm6</t>
+        </is>
+      </c>
+      <c r="H176" s="3" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="inlineStr">
+        <is>
+          <t>Doing outdoor activities or sports</t>
+        </is>
+      </c>
+      <c r="J176" s="3" t="inlineStr">
+        <is>
+          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
+      <c r="K176" s="3" t="inlineStr">
+        <is>
+          <t>matched</t>
+        </is>
+      </c>
+      <c r="L176" s="3" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_5</t>
+          <t>some_apps1_15_TEXT</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -9120,14 +9216,14 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Az eszközöm használata segít elfelejteni a problémáimat</t>
+          <t>Kérjük, jelöld be azt a három alkalmazást vagy szolgáltatást, amelyeket a leggyakrabban használod! - Egyéb: - Text</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr"/>
       <c r="E177" s="2" t="inlineStr"/>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Select the answer that was true for you during the past week. There are no right or wrong answers! - Using my device helps me forget about my problems</t>
+          <t>Please select the three apps or services that you use most often! - Other: - Text</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr"/>
@@ -9144,7 +9240,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_6</t>
+          <t>dasc01:25_2</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -9154,14 +9250,14 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Nem töltök időt a családtagjaimmal, mert szívesebben használom az eszközömet</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Azt érzem, hogy több időt kell töltenem az eszközöm használatával</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr"/>
       <c r="E178" s="2" t="inlineStr"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I do not spend time with my family members because I prefer using my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Select the answer that was true for you during the past week. There are no right or wrong answers! - I feel that I need to spend more time using my device</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr"/>
@@ -9178,7 +9274,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_7</t>
+          <t>dasc01:25_3</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -9188,14 +9284,14 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Egyre több időt töltök az eszközöm használatával</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Feszült leszek, ha nem tudom használni az eszközömet</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr"/>
       <c r="E179" s="2" t="inlineStr"/>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I spend more and more time using my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Select the answer that was true for you during the past week. There are no right or wrong answers! - I become tense if I cannot use my device</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr"/>
@@ -9212,7 +9308,7 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_8</t>
+          <t>dasc01:25_4</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -9222,14 +9318,14 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Ideges leszek, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Hazudok a szüleimnek arról, hogy mennyi időt töltök az eszközöm használatával</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr"/>
       <c r="E180" s="2" t="inlineStr"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I get annoyed when I am asked to stop using my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Select the answer that was true for you during the past week. There are no right or wrong answers! - I lie to my parents about how much time I spend using my device</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr"/>
@@ -9246,7 +9342,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_9</t>
+          <t>dasc01:25_5</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -9256,14 +9352,14 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - A szüleim megpróbálják megakadályozni vagy korlátozni az eszközöm használatát, de nem sikerül nekik</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Az eszközöm használata segít elfelejteni a problémáimat</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr"/>
       <c r="E181" s="2" t="inlineStr"/>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - My parents try to prevent or limit my device use, but they do not succeed</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Select the answer that was true for you during the past week. There are no right or wrong answers! - Using my device helps me forget about my problems</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr"/>
@@ -9280,7 +9376,7 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_11</t>
+          <t>dasc01:25_6</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -9290,14 +9386,14 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Amikor nincs nálam az eszközöm, arra gondolok, amit azon szoktam csinálni (videojátékok, közösségi média, üzenetek stb.)</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Nem töltök időt a családtagjaimmal, mert szívesebben használom az eszközömet</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr"/>
       <c r="E182" s="2" t="inlineStr"/>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - When I don't have my device with me, I think about what I usually do on it (video games, social media, messaging, etc.)</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I do not spend time with my family members because I prefer using my device</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr"/>
@@ -9314,7 +9410,7 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_12</t>
+          <t>dasc01:25_7</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -9324,14 +9420,14 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Feszült vagyok, ha nem tudom használni az eszközömet.</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Egyre több időt töltök az eszközöm használatával</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr"/>
       <c r="E183" s="2" t="inlineStr"/>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I feel tense if I cannot use my device.</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I spend more and more time using my device</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr"/>
@@ -9348,7 +9444,7 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_13</t>
+          <t>dasc01:25_8</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -9358,14 +9454,14 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Konfliktusaim vannak a szüleimmel azzal kapcsolatban, hogy mennyi időt töltök az eszközöm használatával</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Ideges leszek, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr"/>
       <c r="E184" s="2" t="inlineStr"/>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I have conflicts with my parents regarding how much time I spend using my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I get annoyed when I am asked to stop using my device</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr"/>
@@ -9382,7 +9478,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_14</t>
+          <t>dasc01:25_9</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
@@ -9392,14 +9488,14 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Az eszközöm használata a legfontosabb dolog az életemben</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - A szüleim megpróbálják megakadályozni vagy korlátozni az eszközöm használatát, de nem sikerül nekik</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr"/>
       <c r="E185" s="2" t="inlineStr"/>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - Using my device is the most important thing in my life</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - My parents try to prevent or limit my device use, but they do not succeed</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr"/>
@@ -9416,7 +9512,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_15</t>
+          <t>dasc01:25_10</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -9426,31 +9522,47 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Az eszközöm használata élvezetesebb, mint más dolgok</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Kevesebbet alszom az eszközöm használata miatt</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr"/>
       <c r="E186" s="2" t="inlineStr"/>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - Using my device is more enjoyable than other things</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I sleep less because of using my device</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr"/>
-      <c r="H186" s="2" t="inlineStr"/>
-      <c r="I186" s="2" t="inlineStr"/>
-      <c r="J186" s="2" t="inlineStr"/>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>Sleep</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
+        </is>
+      </c>
       <c r="K186" s="2" t="inlineStr">
         <is>
           <t>extra</t>
         </is>
       </c>
-      <c r="L186" s="2" t="inlineStr"/>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>Fallback text match (1.00); Manual fix: DASC item, not smharm1</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_16</t>
+          <t>dasc01:25_11</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -9460,14 +9572,14 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Hazudok a szüleimnek arról, hogy mit csinálok az eszközömön</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Amikor nincs nálam az eszközöm, arra gondolok, amit azon szoktam csinálni (videojátékok, közösségi média, üzenetek stb.)</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr"/>
       <c r="E187" s="2" t="inlineStr"/>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I lie to my parents about what I do on my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - When I don't have my device with me, I think about what I usually do on it (video games, social media, messaging, etc.)</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr"/>
@@ -9484,7 +9596,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_17</t>
+          <t>dasc01:25_12</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -9494,14 +9606,14 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Nem tudom uralni az eszközöm használatát</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Feszült vagyok, ha nem tudom használni az eszközömet.</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr"/>
       <c r="E188" s="2" t="inlineStr"/>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I cannot control my device use</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I feel tense if I cannot use my device.</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr"/>
@@ -9518,7 +9630,7 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_18</t>
+          <t>dasc01:25_13</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -9528,14 +9640,14 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Elvesztettem érdeklődésemet hobbik vagy más tevékenységek iránt, mert inkább az eszközömet használom</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Konfliktusaim vannak a szüleimmel azzal kapcsolatban, hogy mennyi időt töltök az eszközöm használatával</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr"/>
       <c r="E189" s="2" t="inlineStr"/>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I have lost interest in hobbies or other activities because I prefer using my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I have conflicts with my parents regarding how much time I spend using my device</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr"/>
@@ -9552,7 +9664,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_19</t>
+          <t>dasc01:25_14</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -9562,14 +9674,14 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Amikor abbahagyom az eszközöm használatát, nem sokkal később újra elkezdem használni</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Az eszközöm használata a legfontosabb dolog az életemben</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr"/>
       <c r="E190" s="2" t="inlineStr"/>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - When I stop using my device, shortly after I start using it again</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - Using my device is the most important thing in my life</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr"/>
@@ -9586,7 +9698,7 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_20</t>
+          <t>dasc01:25_15</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -9596,14 +9708,14 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Megnézem az eszközöm, amikor házi feladatot vagy más fontos dolgot csinálok</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Az eszközöm használata élvezetesebb, mint más dolgok</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr"/>
       <c r="E191" s="2" t="inlineStr"/>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I check my device when doing homework or other important things</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - Using my device is more enjoyable than other things</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr"/>
@@ -9620,7 +9732,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_21</t>
+          <t>dasc01:25_16</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -9630,14 +9742,14 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Feszült leszek, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Hazudok a szüleimnek arról, hogy mit csinálok az eszközömön</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr"/>
       <c r="E192" s="2" t="inlineStr"/>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I get tense when I am asked to stop using my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I lie to my parents about what I do on my device</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr"/>
@@ -9654,7 +9766,7 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_22</t>
+          <t>dasc01:25_17</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -9664,14 +9776,14 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Összeveszek a szüleimmel, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Nem tudom uralni az eszközöm használatát</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr"/>
       <c r="E193" s="2" t="inlineStr"/>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I get into arguments with my parents when they ask me to stop using my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I cannot control my device use</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr"/>
@@ -9688,7 +9800,7 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_23</t>
+          <t>dasc01:25_18</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -9698,14 +9810,14 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Túl sok pénzt költök az eszközömhöz kapcsolódó dolgokra</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Elvesztettem érdeklődésemet hobbik vagy más tevékenységek iránt, mert inkább az eszközömet használom</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr"/>
       <c r="E194" s="2" t="inlineStr"/>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I spend too much money on things related to my device</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I have lost interest in hobbies or other activities because I prefer using my device</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr"/>
@@ -9722,7 +9834,7 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_24</t>
+          <t>dasc01:25_19</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -9732,14 +9844,14 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Amikor rosszkedvű vagyok, az eszközöm használatától jobb kedvem lesz</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Amikor abbahagyom az eszközöm használatát, nem sokkal később újra elkezdem használni</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr"/>
       <c r="E195" s="2" t="inlineStr"/>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - When I am in a bad mood, using my device puts me in a better mood</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - When I stop using my device, shortly after I start using it again</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr"/>
@@ -9756,7 +9868,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>dasc01:25_25</t>
+          <t>dasc01:25_20</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -9766,14 +9878,14 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Továbbra is használom az eszközöm annak ellenére, hogy az iskolai jegyeim egyre rosszabbak</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Megnézem az eszközöm, amikor házi feladatot vagy más fontos dolgot csinálok</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr"/>
       <c r="E196" s="2" t="inlineStr"/>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I continue to use my device even though my grades at school are getting worse</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I check my device when doing homework or other important things</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr"/>
@@ -9790,7 +9902,7 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>suicide1:5_2</t>
+          <t>dasc01:25_21</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -9800,14 +9912,14 @@
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha? - Voltak ténylegesen olyan gondolataid, hogy megölöd magad?</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Feszült leszek, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr"/>
       <c r="E197" s="2" t="inlineStr"/>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? - Have you actually had thoughts of killing yourself?</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I get tense when I am asked to stop using my device</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr"/>
@@ -9824,7 +9936,7 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>suicide1:5_3</t>
+          <t>dasc01:25_22</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -9834,14 +9946,14 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha? - Gondolkodtál már azon, hogy hogyan ölhetnéd meg magad?</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Összeveszek a szüleimmel, amikor arra kérnek, hogy hagyjam abba az eszközöm használatát</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr"/>
       <c r="E198" s="2" t="inlineStr"/>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? - Have you thought about how you could kill yourself?</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I get into arguments with my parents when they ask me to stop using my device</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr"/>
@@ -9858,7 +9970,7 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>suicide1:5_4</t>
+          <t>dasc01:25_23</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -9868,14 +9980,14 @@
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha? - Elkezdtél-e kidolgozni, esetleg ténylegesen ki is dolgoztál részleteket, hogy hogyan öld meg magad, és szándékodban is állt megvalósítani ezt a tervet?</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Túl sok pénzt költök az eszközömhöz kapcsolódó dolgokra</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr"/>
       <c r="E199" s="2" t="inlineStr"/>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? - Have you started working out or actually worked out details on how to kill yourself, and did you intend to carry out this plan?</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I spend too much money on things related to my device</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr"/>
@@ -9892,7 +10004,7 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>suicide1:5_5</t>
+          <t>dasc01:25_24</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -9902,14 +10014,14 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha? - Kíséreltél már meg öngyilkosságot?</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Amikor rosszkedvű vagyok, az eszközöm használatától jobb kedvem lesz</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr"/>
       <c r="E200" s="2" t="inlineStr"/>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? - Have you ever attempted suicide?</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - When I am in a bad mood, using my device puts me in a better mood</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr"/>
@@ -9926,7 +10038,7 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>suicide6</t>
+          <t>dasc01:25_25</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -9936,14 +10048,14 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Amennyiben kíséreltél már meg öngyilkosságot, hány alkalommal? - Selected Choice</t>
+          <t>Amikor a lenti mondatokban „eszköz” szót olvasol, gondolj minden olyan készülékre, aminek képernyője van: PlayStation, Xbox, okostelefon, tablet, laptop, számítógép, kézi konzol stb. Az „eszközöm használata” azt jelenti, hogy játszol rajta, üzengetsz valakivel, közösségi média oldalakat nézel meg, TikTok vagy YouTube videókat, filmet, sorozatot nézel, stb.  Jelöld be azt a választ, amelyik igaz volt rád az elmúlt héten. Nincsenek jó vagy rossz válaszok! - Továbbra is használom az eszközöm annak ellenére, hogy az iskolai jegyeim egyre rosszabbak</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr"/>
       <c r="E201" s="2" t="inlineStr"/>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>If you have ever attempted suicide, how many times? - Selected Choice</t>
+          <t>When you read the word 'device' in the sentences below, think of any device that has a screen: PlayStation, Xbox, smartphone, tablet, laptop, computer, handheld console, etc. 'Using my device' means playing games on it, messaging someone, checking social media sites, watching TikTok or YouTube videos, movies, series, etc. Mark the answer that was true for you in the past week. There are no right or wrong answers! - I continue to use my device even though my grades at school are getting worse</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr"/>
@@ -9960,7 +10072,7 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>suicide6_1_TEXT</t>
+          <t>suicide1:5_2</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -9970,14 +10082,14 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Amennyiben kíséreltél már meg öngyilkosságot, hány alkalommal? - Ennyi alkalommal: - Text</t>
+          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha? - Voltak ténylegesen olyan gondolataid, hogy megölöd magad?</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr"/>
       <c r="E202" s="2" t="inlineStr"/>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>If you have ever attempted suicide, how many times? - This many times: - Text</t>
+          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? - Have you actually had thoughts of killing yourself?</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr"/>
@@ -9994,7 +10106,7 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse1:3_1</t>
+          <t>suicide1:5_3</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -10004,14 +10116,14 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi dohánytermékeket az elmúlt 30 nap során? - Cigaretta</t>
+          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha? - Gondolkodtál már azon, hogy hogyan ölhetnéd meg magad?</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr"/>
       <c r="E203" s="2" t="inlineStr"/>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>How often did you use the following tobacco products in the past 30 days? - Cigarettes</t>
+          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? - Have you thought about how you could kill yourself?</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr"/>
@@ -10028,7 +10140,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse1:3_2</t>
+          <t>suicide1:5_4</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -10038,14 +10150,14 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi dohánytermékeket az elmúlt 30 nap során? - E-cigaretta (pl. iqos, elfbar, poco)</t>
+          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha? - Elkezdtél-e kidolgozni, esetleg ténylegesen ki is dolgoztál részleteket, hogy hogyan öld meg magad, és szándékodban is állt megvalósítani ezt a tervet?</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr"/>
       <c r="E204" s="2" t="inlineStr"/>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>How often did you use the following tobacco products in the past 30 days? - E-cigarettes (e.g. iqos, elfbar, poco)</t>
+          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? - Have you started working out or actually worked out details on how to kill yourself, and did you intend to carry out this plan?</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr"/>
@@ -10062,7 +10174,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse1:3_3</t>
+          <t>suicide1:5_5</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -10072,14 +10184,14 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi dohánytermékeket az elmúlt 30 nap során? - Szájba helyezett dohány (snus)</t>
+          <t>Tapasztaltad vagy tetted-e az alábbiak közül bármelyiket az elmúlt 30 napban vagy életedben valaha? - Kíséreltél már meg öngyilkosságot?</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr"/>
       <c r="E205" s="2" t="inlineStr"/>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>How often did you use the following tobacco products in the past 30 days? - Oral tobacco (snus)</t>
+          <t>Have you experienced or done any of the following in the past 30 days or ever in your life? - Have you ever attempted suicide?</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr"/>
@@ -10096,7 +10208,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse4:6_1</t>
+          <t>suicide6</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -10106,14 +10218,14 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi dohánytermékeket az életed során? - Cigaretta</t>
+          <t>Amennyiben kíséreltél már meg öngyilkosságot, hány alkalommal? - Selected Choice</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr"/>
       <c r="E206" s="2" t="inlineStr"/>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>How often did you use the following tobacco products in your lifetime? - Cigarettes</t>
+          <t>If you have ever attempted suicide, how many times? - Selected Choice</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr"/>
@@ -10130,7 +10242,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse4:6_2</t>
+          <t>suicide6_1_TEXT</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -10140,14 +10252,14 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi dohánytermékeket az életed során? - E-cigaretta (pl. iqos, elfbar, poco)</t>
+          <t>Amennyiben kíséreltél már meg öngyilkosságot, hány alkalommal? - Ennyi alkalommal: - Text</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr"/>
       <c r="E207" s="2" t="inlineStr"/>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>How often did you use the following tobacco products in your lifetime? - E-cigarettes (e.g. iqos, elfbar, poco)</t>
+          <t>If you have ever attempted suicide, how many times? - This many times: - Text</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr"/>
@@ -10164,7 +10276,7 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse4:6_3</t>
+          <t>sub_abuse1:3_1</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -10174,14 +10286,14 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi dohánytermékeket az életed során? - Szájba helyezett dohány (snus)</t>
+          <t>Milyen gyakran használtad az alábbi dohánytermékeket az elmúlt 30 nap során? - Cigaretta</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr"/>
       <c r="E208" s="2" t="inlineStr"/>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>How often did you use the following tobacco products in your lifetime? - Oral tobacco (snus)</t>
+          <t>How often did you use the following tobacco products in the past 30 days? - Cigarettes</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr"/>
@@ -10198,7 +10310,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse7</t>
+          <t>sub_abuse1:3_2</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -10208,14 +10320,14 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran fogyasztottál alkoholos italokat (pl. sör, alkoholos üdítőital, bor, rövid italok/shotok) az elmúlt 30 nap során?</t>
+          <t>Milyen gyakran használtad az alábbi dohánytermékeket az elmúlt 30 nap során? - E-cigaretta (pl. iqos, elfbar, poco)</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr"/>
       <c r="E209" s="2" t="inlineStr"/>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>How often did you consume alcoholic beverages (e.g. beer, alcopops, wine, spirits/shots) in the past 30 days?</t>
+          <t>How often did you use the following tobacco products in the past 30 days? - E-cigarettes (e.g. iqos, elfbar, poco)</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr"/>
@@ -10232,7 +10344,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse9</t>
+          <t>sub_abuse1:3_3</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -10242,14 +10354,14 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran rúgtál be az elmúlt 30 nap során?</t>
+          <t>Milyen gyakran használtad az alábbi dohánytermékeket az elmúlt 30 nap során? - Szájba helyezett dohány (snus)</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr"/>
       <c r="E210" s="2" t="inlineStr"/>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>How often did you get drunk in the past 30 days?</t>
+          <t>How often did you use the following tobacco products in the past 30 days? - Oral tobacco (snus)</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr"/>
@@ -10266,7 +10378,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse10</t>
+          <t>sub_abuse4:6_1</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -10276,14 +10388,14 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran rúgtál be életed során?</t>
+          <t>Milyen gyakran használtad az alábbi dohánytermékeket az életed során? - Cigaretta</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr"/>
       <c r="E211" s="2" t="inlineStr"/>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>How often did you get drunk in your lifetime?</t>
+          <t>How often did you use the following tobacco products in your lifetime? - Cigarettes</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr"/>
@@ -10300,7 +10412,7 @@
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse12</t>
+          <t>sub_abuse4:6_2</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -10310,14 +10422,14 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtál életed során olyan vényköteles gyógyszert, amelyet nem neked írtak fel (pl. nyugtatók, stimulánsok)?</t>
+          <t>Milyen gyakran használtad az alábbi dohánytermékeket az életed során? - E-cigaretta (pl. iqos, elfbar, poco)</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr"/>
       <c r="E212" s="2" t="inlineStr"/>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>How often in your lifetime have you used prescription medication that was not prescribed to you (e.g. sedatives, stimulants)?</t>
+          <t>How often did you use the following tobacco products in your lifetime? - E-cigarettes (e.g. iqos, elfbar, poco)</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr"/>
@@ -10334,7 +10446,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse13</t>
+          <t>sub_abuse4:6_3</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -10344,14 +10456,14 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtál életed során olyan tudatmódosító szert, amelyet nem tekintenek kábítószernek (például ragasztót, gázt, festéket vagy patront)?</t>
+          <t>Milyen gyakran használtad az alábbi dohánytermékeket az életed során? - Szájba helyezett dohány (snus)</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr"/>
       <c r="E213" s="2" t="inlineStr"/>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>How often in your lifetime have you used a mind-altering substance not considered a drug (such as glue, gas, paint, or cartridges)?</t>
+          <t>How often did you use the following tobacco products in your lifetime? - Oral tobacco (snus)</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr"/>
@@ -10368,7 +10480,7 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse14</t>
+          <t>sub_abuse7</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -10378,14 +10490,14 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Használtál valaha valamilyen drogot?</t>
+          <t>Milyen gyakran fogyasztottál alkoholos italokat (pl. sör, alkoholos üdítőital, bor, rövid italok/shotok) az elmúlt 30 nap során?</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr"/>
       <c r="E214" s="2" t="inlineStr"/>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>Have you ever used any drugs?</t>
+          <t>How often did you consume alcoholic beverages (e.g. beer, alcopops, wine, spirits/shots) in the past 30 days?</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr"/>
@@ -10402,7 +10514,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse15:18_1</t>
+          <t>sub_abuse9</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -10412,14 +10524,14 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során? - Kábítószer cigarettában elszívva</t>
+          <t>Milyen gyakran rúgtál be az elmúlt 30 nap során?</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr"/>
       <c r="E215" s="2" t="inlineStr"/>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>How often did you use the following drugs in the past 30 days? - Drugs smoked in a cigarette</t>
+          <t>How often did you get drunk in the past 30 days?</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr"/>
@@ -10436,7 +10548,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse15:18_2</t>
+          <t>sub_abuse10</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -10446,14 +10558,14 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során? - Kábítószer szájon át bevéve</t>
+          <t>Milyen gyakran rúgtál be életed során?</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr"/>
       <c r="E216" s="2" t="inlineStr"/>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>How often did you use the following drugs in the past 30 days? - Drugs taken orally</t>
+          <t>How often did you get drunk in your lifetime?</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr"/>
@@ -10470,7 +10582,7 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse15:18_3</t>
+          <t>sub_abuse12</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -10480,14 +10592,14 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során? - Kábítószer orrba felszippantva</t>
+          <t>Milyen gyakran használtál életed során olyan vényköteles gyógyszert, amelyet nem neked írtak fel (pl. nyugtatók, stimulánsok)?</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr"/>
       <c r="E217" s="2" t="inlineStr"/>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>How often have you used the following drugs during the past 30 days? - Drugs snorted through the nose</t>
+          <t>How often in your lifetime have you used prescription medication that was not prescribed to you (e.g. sedatives, stimulants)?</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr"/>
@@ -10504,7 +10616,7 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse15:18_4</t>
+          <t>sub_abuse13</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -10514,14 +10626,14 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során? - Kábítószer intravénásan (érbe) befecskendezve</t>
+          <t>Milyen gyakran használtál életed során olyan tudatmódosító szert, amelyet nem tekintenek kábítószernek (például ragasztót, gázt, festéket vagy patront)?</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr"/>
       <c r="E218" s="2" t="inlineStr"/>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>How often have you used the following drugs during the past 30 days? - Drugs injected intravenously (into a vein)</t>
+          <t>How often in your lifetime have you used a mind-altering substance not considered a drug (such as glue, gas, paint, or cartridges)?</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr"/>
@@ -10538,7 +10650,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse19:22_1</t>
+          <t>sub_abuse14</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -10548,14 +10660,14 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi kábítószereket életed során? - Kábítószer cigarettában elszívva</t>
+          <t>Használtál valaha valamilyen drogot?</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr"/>
       <c r="E219" s="2" t="inlineStr"/>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>How often have you used the following drugs during your lifetime? - Drugs smoked in a cigarette</t>
+          <t>Have you ever used any drugs?</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr"/>
@@ -10572,7 +10684,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse19:22_2</t>
+          <t>sub_abuse15:18_1</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -10582,14 +10694,14 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi kábítószereket életed során? - Kábítószer szájon át bevéve</t>
+          <t>Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során? - Kábítószer cigarettában elszívva</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr"/>
       <c r="E220" s="2" t="inlineStr"/>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>How often have you used the following drugs during your lifetime? - Drugs taken orally</t>
+          <t>How often did you use the following drugs in the past 30 days? - Drugs smoked in a cigarette</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr"/>
@@ -10606,7 +10718,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse19:22_3</t>
+          <t>sub_abuse15:18_2</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -10616,14 +10728,14 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi kábítószereket életed során? - Kábítószer orrba felszippantva</t>
+          <t>Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során? - Kábítószer szájon át bevéve</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr"/>
       <c r="E221" s="2" t="inlineStr"/>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>How often have you used the following drugs during your lifetime? - Drugs snorted through the nose</t>
+          <t>How often did you use the following drugs in the past 30 days? - Drugs taken orally</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr"/>
@@ -10640,7 +10752,7 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>sub_abuse19:22_4</t>
+          <t>sub_abuse15:18_3</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -10650,14 +10762,14 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Milyen gyakran használtad az alábbi kábítószereket életed során? - Kábítószer intravénásan (érbe) befecskendezve</t>
+          <t>Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során? - Kábítószer orrba felszippantva</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr"/>
       <c r="E222" s="2" t="inlineStr"/>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>How often have you used the following drugs during your lifetime? - Drugs injected intravenously (into a vein)</t>
+          <t>How often have you used the following drugs during the past 30 days? - Drugs snorted through the nose</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr"/>
@@ -10674,7 +10786,7 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>repa1:8_2</t>
+          <t>sub_abuse15:18_4</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -10684,14 +10796,14 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - Jól kijövök a szüleimmel</t>
+          <t>Milyen gyakran használtad az alábbi kábítószereket az elmúlt 30 nap során? - Kábítószer intravénásan (érbe) befecskendezve</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr"/>
       <c r="E223" s="2" t="inlineStr"/>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - I get along well with my parents</t>
+          <t>How often have you used the following drugs during the past 30 days? - Drugs injected intravenously (into a vein)</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr"/>
@@ -10708,7 +10820,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>repa1:8_3</t>
+          <t>sub_abuse19:22_1</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -10718,14 +10830,14 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - A szüleim kedvelnek engem</t>
+          <t>Milyen gyakran használtad az alábbi kábítószereket életed során? - Kábítószer cigarettában elszívva</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr"/>
       <c r="E224" s="2" t="inlineStr"/>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - My parents like me</t>
+          <t>How often have you used the following drugs during your lifetime? - Drugs smoked in a cigarette</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr"/>
@@ -10742,7 +10854,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>repa1:8_4</t>
+          <t>sub_abuse19:22_2</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -10752,14 +10864,14 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - Kedvelem a szüleimet</t>
+          <t>Milyen gyakran használtad az alábbi kábítószereket életed során? - Kábítószer szájon át bevéve</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr"/>
       <c r="E225" s="2" t="inlineStr"/>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - I like my parents</t>
+          <t>How often have you used the following drugs during your lifetime? - Drugs taken orally</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr"/>
@@ -10776,7 +10888,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>repa1:8_5</t>
+          <t>sub_abuse19:22_3</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -10786,14 +10898,14 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - A szüleim kritizálnak</t>
+          <t>Milyen gyakran használtad az alábbi kábítószereket életed során? - Kábítószer orrba felszippantva</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr"/>
       <c r="E226" s="2" t="inlineStr"/>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - My parents criticize me</t>
+          <t>How often have you used the following drugs during your lifetime? - Drugs snorted through the nose</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr"/>
@@ -10810,7 +10922,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>repa1:8_6</t>
+          <t>sub_abuse19:22_4</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -10820,14 +10932,14 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - A szüleim idegesítenek</t>
+          <t>Milyen gyakran használtad az alábbi kábítószereket életed során? - Kábítószer intravénásan (érbe) befecskendezve</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr"/>
       <c r="E227" s="2" t="inlineStr"/>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - My parents annoy me</t>
+          <t>How often have you used the following drugs during your lifetime? - Drugs injected intravenously (into a vein)</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr"/>
@@ -10844,7 +10956,7 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>repa1:8_7</t>
+          <t>repa1:8_2</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -10854,14 +10966,14 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - A szüleim megbántanak engem</t>
+          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - Jól kijövök a szüleimmel</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr"/>
       <c r="E228" s="2" t="inlineStr"/>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - My parents hurt my feelings</t>
+          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - I get along well with my parents</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr"/>
@@ -10878,7 +10990,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>repa1:8_8</t>
+          <t>repa1:8_3</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -10888,14 +11000,14 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - Vitatkozunk a szüleimmel</t>
+          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - A szüleim kedvelnek engem</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr"/>
       <c r="E229" s="2" t="inlineStr"/>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - We argue with my parents</t>
+          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - My parents like me</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr"/>
@@ -10912,7 +11024,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>refr1:5_2</t>
+          <t>repa1:8_4</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -10922,14 +11034,14 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Mennyire érvényesek rád az alábbi állítások? - Sok barátom van</t>
+          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - Kedvelem a szüleimet</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr"/>
       <c r="E230" s="2" t="inlineStr"/>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>To what extent do the following statements apply to you? - I have many friends</t>
+          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - I like my parents</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr"/>
@@ -10946,7 +11058,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>refr1:5_3</t>
+          <t>repa1:8_5</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -10956,14 +11068,14 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Mennyire érvényesek rád az alábbi állítások? - A többi fiatal nehéznek találja, hogy kedveljen engem</t>
+          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - A szüleim kritizálnak</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr"/>
       <c r="E231" s="2" t="inlineStr"/>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>To what extent do the following statements apply to you? - Other young people find it difficult to like me</t>
+          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - My parents criticize me</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr"/>
@@ -10980,7 +11092,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>refr1:5_4</t>
+          <t>repa1:8_6</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -10990,14 +11102,14 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Mennyire érvényesek rád az alábbi állítások? - Népszerű vagyok a többi fiatal körében</t>
+          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - A szüleim idegesítenek</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr"/>
       <c r="E232" s="2" t="inlineStr"/>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>To what extent do the following statements apply to you? - I am popular among other young people</t>
+          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - My parents annoy me</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr"/>
@@ -11014,7 +11126,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>refr1:5_5</t>
+          <t>repa1:8_7</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -11024,14 +11136,14 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>Mennyire érvényesek rád az alábbi állítások? - Érzem, hogy mások elfogadnak</t>
+          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - A szüleim megbántanak engem</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr"/>
       <c r="E233" s="2" t="inlineStr"/>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>To what extent do the following statements apply to you? - I feel accepted by others</t>
+          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - My parents hurt my feelings</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr"/>
@@ -11048,7 +11160,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>leisure1:5_2</t>
+          <t>repa1:8_8</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -11058,14 +11170,14 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket? - Edzeni (pl. foci, kézilabda, síelés, futás, tánc, torna)</t>
+          <t>Alább található néhány állítás arról, hogyan kommunikálnak a fiatalok a szüleikkel. Kérjük, jelöld be, milyen gyakran érzed az alábbiakat a családodban. - Vitatkozunk a szüleimmel</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr"/>
       <c r="E234" s="2" t="inlineStr"/>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>Outside of school: In an average week, on how many days do you usually do the following? - Work out / exercise (e.g., football, handball, skiing, running, dance, gymnastics)</t>
+          <t>Below are some statements about how young people communicate with their parents. Please indicate how often you feel the following in your family. - We argue with my parents</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr"/>
@@ -11082,7 +11194,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>leisure1:5_3</t>
+          <t>refr1:5_2</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -11092,14 +11204,14 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket? - Részt venni más szervezett tevékenységekben (pl. színház, zene, cserkészkedés)</t>
+          <t>Mennyire érvényesek rád az alábbi állítások? - Sok barátom van</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr"/>
       <c r="E235" s="2" t="inlineStr"/>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>Outside of school: In an average week, on how many days do you usually do the following? - Participate in other organized activities (e.g., theater, music, scouting)</t>
+          <t>To what extent do the following statements apply to you? - I have many friends</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr"/>
@@ -11116,7 +11228,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>leisure1:5_4</t>
+          <t>refr1:5_3</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -11126,14 +11238,14 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket? - Egész délután és este otthon maradni</t>
+          <t>Mennyire érvényesek rád az alábbi állítások? - A többi fiatal nehéznek találja, hogy kedveljen engem</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr"/>
       <c r="E236" s="2" t="inlineStr"/>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>Outside of school: In an average week, on how many days do you usually do the following? - Stay at home the whole afternoon and evening</t>
+          <t>To what extent do the following statements apply to you? - Other young people find it difficult to like me</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr"/>
@@ -11150,7 +11262,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>leisure1:5_5</t>
+          <t>refr1:5_4</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -11160,14 +11272,14 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket? - Könyveket olvasni vagy hangoskönyveket hallgatni</t>
+          <t>Mennyire érvényesek rád az alábbi állítások? - Népszerű vagyok a többi fiatal körében</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr"/>
       <c r="E237" s="2" t="inlineStr"/>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>Outside of school: On an average week, how many days do you do the following? : Reading books or listening to audiobooks</t>
+          <t>To what extent do the following statements apply to you? - I am popular among other young people</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr"/>
@@ -11184,7 +11296,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>physact1</t>
+          <t>refr1:5_5</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -11194,14 +11306,14 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Az iskolán kívül: Hetente körülbelül hány órát sportolsz úgy vagy végzel olyan fizikai tevékenységet (pl. foci, kézilabda, futás, torna, tánc stb.), amelyben kifulladsz vagy izzadsz? - Selected Choice</t>
+          <t>Mennyire érvényesek rád az alábbi állítások? - Érzem, hogy mások elfogadnak</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr"/>
       <c r="E238" s="2" t="inlineStr"/>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>Outside of school: Approximately how many hours a week do you do sports or engage in physical activity (e.g., soccer, handball, running, gymnastics, dance, etc.) that makes you out of breath or sweat? - Selected Choice</t>
+          <t>To what extent do the following statements apply to you? - I feel accepted by others</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr"/>
@@ -11218,7 +11330,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>physact1_1_TEXT</t>
+          <t>leisure1:5_2</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -11228,14 +11340,14 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Az iskolán kívül: Hetente körülbelül hány órát sportolsz úgy vagy végzel olyan fizikai tevékenységet (pl. foci, kézilabda, futás, torna, tánc stb.), amelyben kifulladsz vagy izzadsz? - Ennyi órát: - Text</t>
+          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket? - Edzeni (pl. foci, kézilabda, síelés, futás, tánc, torna)</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr"/>
       <c r="E239" s="2" t="inlineStr"/>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>Outside of school: Approximately how many hours a week do you do sports or engage in physical activity (e.g., soccer, handball, running, gymnastics, dance, etc.) that makes you out of breath or sweat? - This many hours: - Text</t>
+          <t>Outside of school: In an average week, on how many days do you usually do the following? - Work out / exercise (e.g., football, handball, skiing, running, dance, gymnastics)</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr"/>
@@ -11252,7 +11364,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>activity_week1:5_2</t>
+          <t>leisure1:5_3</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -11262,14 +11374,14 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel? - Házi feladat elkészítése</t>
+          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket? - Részt venni más szervezett tevékenységekben (pl. színház, zene, cserkészkedés)</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr"/>
       <c r="E240" s="2" t="inlineStr"/>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>On an average weekday, how much time do you spend on the following activities? : Doing homework</t>
+          <t>Outside of school: In an average week, on how many days do you usually do the following? - Participate in other organized activities (e.g., theater, music, scouting)</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr"/>
@@ -11286,7 +11398,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>activity_week1:5_3</t>
+          <t>leisure1:5_4</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -11296,14 +11408,14 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel? - Játék PC-n (asztali számítógépen), TV-n, tableten, telefonon stb.</t>
+          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket? - Egész délután és este otthon maradni</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr"/>
       <c r="E241" s="2" t="inlineStr"/>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>On an average weekday, how much time do you spend on the following activities? : Playing games on PC (desktop computer), TV, tablet, phone, etc.</t>
+          <t>Outside of school: In an average week, on how many days do you usually do the following? - Stay at home the whole afternoon and evening</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr"/>
@@ -11320,7 +11432,7 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>activity_week1:5_4</t>
+          <t>leisure1:5_5</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -11330,14 +11442,14 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel? - Leülni a számítógép elé, vagy leülni/lefeküdni telefonnal vagy táblagéppel (tevékenységtől függetlenül)</t>
+          <t>Az iskolán kívül: Egy átlagos héten hány napon szoktad csinálni a következőket? - Könyveket olvasni vagy hangoskönyveket hallgatni</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr"/>
       <c r="E242" s="2" t="inlineStr"/>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>On an average weekday, how much time do you spend on the following activities? : Sitting in front of the computer, or sitting/lying down with a phone or tablet (regardless of activity)</t>
+          <t>Outside of school: On an average week, how many days do you do the following? : Reading books or listening to audiobooks</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr"/>
@@ -11354,7 +11466,7 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>activity_week1:5_5</t>
+          <t>physact1</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -11364,14 +11476,14 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel? - A közösségi media aktív használata (nem csak bejelentkezve lenni)</t>
+          <t>Az iskolán kívül: Hetente körülbelül hány órát sportolsz úgy vagy végzel olyan fizikai tevékenységet (pl. foci, kézilabda, futás, torna, tánc stb.), amelyben kifulladsz vagy izzadsz? - Selected Choice</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr"/>
       <c r="E243" s="2" t="inlineStr"/>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>On an average weekday, how much time do you spend on the following activities? : Active use of social media (not just being logged in)</t>
+          <t>Outside of school: Approximately how many hours a week do you do sports or engage in physical activity (e.g., soccer, handball, running, gymnastics, dance, etc.) that makes you out of breath or sweat? - Selected Choice</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr"/>
@@ -11388,7 +11500,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>activity_weekend1:5_2</t>
+          <t>physact1_1_TEXT</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -11398,14 +11510,14 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel? - Házi feladat elkészítése</t>
+          <t>Az iskolán kívül: Hetente körülbelül hány órát sportolsz úgy vagy végzel olyan fizikai tevékenységet (pl. foci, kézilabda, futás, torna, tánc stb.), amelyben kifulladsz vagy izzadsz? - Ennyi órát: - Text</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr"/>
       <c r="E244" s="2" t="inlineStr"/>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>On an average weekend day or holiday, how much time do you spend on the following activities? : Doing homework</t>
+          <t>Outside of school: Approximately how many hours a week do you do sports or engage in physical activity (e.g., soccer, handball, running, gymnastics, dance, etc.) that makes you out of breath or sweat? - This many hours: - Text</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr"/>
@@ -11422,7 +11534,7 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>activity_weekend1:5_3</t>
+          <t>activity_week1:5_2</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -11432,14 +11544,14 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel? - Játék PC-n (asztali számítógépen), TV-n, tableten, telefonon stb.</t>
+          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel? - Házi feladat elkészítése</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr"/>
       <c r="E245" s="2" t="inlineStr"/>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>On an average weekend day or holiday, how much time do you spend on the following activities? : Playing games on PC (desktop computer), TV, tablet, phone, etc.</t>
+          <t>On an average weekday, how much time do you spend on the following activities? : Doing homework</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr"/>
@@ -11456,7 +11568,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>activity_weekend1:5_4</t>
+          <t>activity_week1:5_3</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -11466,14 +11578,14 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel? - Leülni a számítógép elé, vagy leülni/lefeküdni telefonnal vagy táblagéppel (tevékenységtől függetlenül)</t>
+          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel? - Játék PC-n (asztali számítógépen), TV-n, tableten, telefonon stb.</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr"/>
       <c r="E246" s="2" t="inlineStr"/>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>On an average weekend day or holiday, how much time do you spend on the following activities? : Sitting in front of the computer, or sitting/lying down with a phone or tablet (regardless of activity)</t>
+          <t>On an average weekday, how much time do you spend on the following activities? : Playing games on PC (desktop computer), TV, tablet, phone, etc.</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr"/>
@@ -11490,7 +11602,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>activity_weekend1:5_5</t>
+          <t>activity_week1:5_4</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -11500,14 +11612,14 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel? - A közösségi media aktív használata (nem csak bejelentkezve lenni)</t>
+          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel? - Leülni a számítógép elé, vagy leülni/lefeküdni telefonnal vagy táblagéppel (tevékenységtől függetlenül)</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr"/>
       <c r="E247" s="2" t="inlineStr"/>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>On an average weekend day or holiday, how much time do you spend on the following activities? : Active use of social media (not just being logged in)</t>
+          <t>On an average weekday, how much time do you spend on the following activities? : Sitting in front of the computer, or sitting/lying down with a phone or tablet (regardless of activity)</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr"/>
@@ -11524,7 +11636,7 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>training2</t>
+          <t>activity_week1:5_5</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -11534,14 +11646,14 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Hány évesen hagytad abba a szervezett sportolást? - Selected Choice</t>
+          <t>Egy átlagos hétköznapon mennyi időt töltesz a következő tevékenységekkel? - A közösségi media aktív használata (nem csak bejelentkezve lenni)</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr"/>
       <c r="E248" s="2" t="inlineStr"/>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>At what age did you quit organized sports? - Selected Choice</t>
+          <t>On an average weekday, how much time do you spend on the following activities? : Active use of social media (not just being logged in)</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr"/>
@@ -11558,7 +11670,7 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>training2_1_TEXT</t>
+          <t>activity_weekend1:5_2</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -11568,14 +11680,14 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>Hány évesen hagytad abba a szervezett sportolást? - Ennyi évesen: - Text</t>
+          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel? - Házi feladat elkészítése</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr"/>
       <c r="E249" s="2" t="inlineStr"/>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>At what age did you quit organized sports? - At this age: - Text</t>
+          <t>On an average weekend day or holiday, how much time do you spend on the following activities? : Doing homework</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr"/>
@@ -11592,7 +11704,7 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>school1:11_2</t>
+          <t>activity_weekend1:5_3</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -11602,14 +11714,14 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - A tanáraim törődnek velem.</t>
+          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel? - Játék PC-n (asztali számítógépen), TV-n, tableten, telefonon stb.</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr"/>
       <c r="E250" s="2" t="inlineStr"/>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - My teachers care about me.</t>
+          <t>On an average weekend day or holiday, how much time do you spend on the following activities? : Playing games on PC (desktop computer), TV, tablet, phone, etc.</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr"/>
@@ -11626,7 +11738,7 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>school1:11_3</t>
+          <t>activity_weekend1:5_4</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -11636,14 +11748,14 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Úgy érzem, beilleszkedem a diákok közé az iskolában.</t>
+          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel? - Leülni a számítógép elé, vagy leülni/lefeküdni telefonnal vagy táblagéppel (tevékenységtől függetlenül)</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr"/>
       <c r="E251" s="2" t="inlineStr"/>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - I feel that I fit in among the students at school.</t>
+          <t>On an average weekend day or holiday, how much time do you spend on the following activities? : Sitting in front of the computer, or sitting/lying down with a phone or tablet (regardless of activity)</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr"/>
@@ -11660,7 +11772,7 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>school1:11_4</t>
+          <t>activity_weekend1:5_5</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -11670,14 +11782,14 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Unatkozom az iskolában.</t>
+          <t>Egy átlagos hétvégi napon vagy ünnepnapon mennyi időt töltesz a következő tevékenységekkel? - A közösségi media aktív használata (nem csak bejelentkezve lenni)</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr"/>
       <c r="E252" s="2" t="inlineStr"/>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - I am bored at school.</t>
+          <t>On an average weekend day or holiday, how much time do you spend on the following activities? : Active use of social media (not just being logged in)</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr"/>
@@ -11694,7 +11806,7 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>school1:11_5</t>
+          <t>training2</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
@@ -11704,14 +11816,14 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Sokan azt várják tőlem, hogy jól teljesítsek az iskolában.</t>
+          <t>Hány évesen hagytad abba a szervezett sportolást? - Selected Choice</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr"/>
       <c r="E253" s="2" t="inlineStr"/>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - Many people expect me to do well at school.</t>
+          <t>At what age did you quit organized sports? - Selected Choice</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr"/>
@@ -11728,7 +11840,7 @@
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>school1:11_6</t>
+          <t>training2_1_TEXT</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
@@ -11738,14 +11850,14 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Gyakran rettegek iskolába menni.</t>
+          <t>Hány évesen hagytad abba a szervezett sportolást? - Ennyi évesen: - Text</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr"/>
       <c r="E254" s="2" t="inlineStr"/>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - I often dread going to school.</t>
+          <t>At what age did you quit organized sports? - At this age: - Text</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr"/>
@@ -11762,7 +11874,7 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>school1:11_7</t>
+          <t>school1:11_2</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -11772,14 +11884,14 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - A hétvégéket gyakran iskolai munkával kell töltenem.</t>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - A tanáraim törődnek velem.</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr"/>
       <c r="E255" s="2" t="inlineStr"/>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - I often have to spend weekends doing schoolwork.</t>
+          <t>Please indicate how much you agree with the following statements! - My teachers care about me.</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr"/>
@@ -11796,7 +11908,7 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>school1:11_8</t>
+          <t>school1:11_3</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -11806,14 +11918,14 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Túl sok a zaj és a rendbontás az órákon.</t>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Úgy érzem, beilleszkedem a diákok közé az iskolában.</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr"/>
       <c r="E256" s="2" t="inlineStr"/>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - There is too much noise and disruption during classes.</t>
+          <t>Please indicate how much you agree with the following statements! - I feel that I fit in among the students at school.</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr"/>
@@ -11830,7 +11942,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>school1:11_9</t>
+          <t>school1:11_4</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -11840,14 +11952,14 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Az iskolában sok az elvesztegetett idő.</t>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Unatkozom az iskolában.</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr"/>
       <c r="E257" s="2" t="inlineStr"/>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - A lot of time is wasted at school.</t>
+          <t>Please indicate how much you agree with the following statements! - I am bored at school.</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr"/>
@@ -11864,7 +11976,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>school1:11_10</t>
+          <t>school1:11_5</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -11874,14 +11986,14 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Sok érdekes dolgot tanulunk az iskolában.</t>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Sokan azt várják tőlem, hogy jól teljesítsek az iskolában.</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr"/>
       <c r="E258" s="2" t="inlineStr"/>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - We learn many interesting things at school.</t>
+          <t>Please indicate how much you agree with the following statements! - Many people expect me to do well at school.</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr"/>
@@ -11898,7 +12010,7 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>school1:11_11</t>
+          <t>school1:11_6</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
@@ -11908,14 +12020,14 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Fontos a jó jegyek megszerzése.</t>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Gyakran rettegek iskolába menni.</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr"/>
       <c r="E259" s="2" t="inlineStr"/>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>Please indicate how much you agree with the following statements! - Getting good grades is important.</t>
+          <t>Please indicate how much you agree with the following statements! - I often dread going to school.</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr"/>
@@ -11932,7 +12044,7 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>school_stress1:3_2</t>
+          <t>school1:11_7</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
@@ -11942,14 +12054,14 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>Iskolai stressz - Kimerültnek érzem magam az iskolai feladatok miatt.</t>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - A hétvégéket gyakran iskolai munkával kell töltenem.</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr"/>
       <c r="E260" s="2" t="inlineStr"/>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>School stress - I feel exhausted because of school tasks.</t>
+          <t>Please indicate how much you agree with the following statements! - I often have to spend weekends doing schoolwork.</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr"/>
@@ -11966,7 +12078,7 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>school_stress1:3_3</t>
+          <t>school1:11_8</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -11976,14 +12088,14 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>Iskolai stressz - Több iskolai feladatom van, mint amennyit kezelni tudok.</t>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Túl sok a zaj és a rendbontás az órákon.</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr"/>
       <c r="E261" s="2" t="inlineStr"/>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>School stress - I have more school tasks than I can handle.</t>
+          <t>Please indicate how much you agree with the following statements! - There is too much noise and disruption during classes.</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr"/>
@@ -12000,7 +12112,7 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>schooltype_1_TEXT</t>
+          <t>school1:11_9</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -12010,14 +12122,14 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>Melyik felsőoktatási intézménybe, és milyen szakra jársz? - Az alábbi intézménybe és szakra járok: - Text</t>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Az iskolában sok az elvesztegetett idő.</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr"/>
       <c r="E262" s="2" t="inlineStr"/>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>Which higher education institution and which program do you attend? - I attend the following institution and program: - Text</t>
+          <t>Please indicate how much you agree with the following statements! - A lot of time is wasted at school.</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr"/>
@@ -12032,254 +12144,174 @@
       <c r="L262" s="2" t="inlineStr"/>
     </row>
     <row r="263">
-      <c r="A263" s="3" t="inlineStr">
-        <is>
-          <t>some_use1:6_2</t>
-        </is>
-      </c>
-      <c r="B263" s="3" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C263" s="3" t="inlineStr">
-        <is>
-          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Iskolai feladatok</t>
-        </is>
-      </c>
-      <c r="D263" s="3" t="inlineStr"/>
-      <c r="E263" s="3" t="inlineStr"/>
-      <c r="F263" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Schoolwork | Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="G263" s="3" t="inlineStr">
-        <is>
-          <t>smharm2</t>
-        </is>
-      </c>
-      <c r="H263" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
-        </is>
-      </c>
-      <c r="I263" s="3" t="inlineStr">
-        <is>
-          <t>Schoolwork</t>
-        </is>
-      </c>
-      <c r="J263" s="3" t="inlineStr">
-        <is>
-          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="K263" s="3" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="L263" s="3" t="inlineStr"/>
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>school1:11_10</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Sok érdekes dolgot tanulunk az iskolában.</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr"/>
+      <c r="E263" s="2" t="inlineStr"/>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>Please indicate how much you agree with the following statements! - We learn many interesting things at school.</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr"/>
+      <c r="H263" s="2" t="inlineStr"/>
+      <c r="I263" s="2" t="inlineStr"/>
+      <c r="J263" s="2" t="inlineStr"/>
+      <c r="K263" s="2" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="L263" s="2" t="inlineStr"/>
     </row>
     <row r="264">
-      <c r="A264" s="3" t="inlineStr">
-        <is>
-          <t>some_use1:6_3</t>
-        </is>
-      </c>
-      <c r="B264" s="3" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C264" s="3" t="inlineStr">
-        <is>
-          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Önbecsülés/mentális egészség</t>
-        </is>
-      </c>
-      <c r="D264" s="3" t="inlineStr"/>
-      <c r="E264" s="3" t="inlineStr"/>
-      <c r="F264" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Self-esteem/mental health | Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="G264" s="3" t="inlineStr">
-        <is>
-          <t>smharm3</t>
-        </is>
-      </c>
-      <c r="H264" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
-        </is>
-      </c>
-      <c r="I264" s="3" t="inlineStr">
-        <is>
-          <t>Self-esteem/mental health</t>
-        </is>
-      </c>
-      <c r="J264" s="3" t="inlineStr">
-        <is>
-          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="K264" s="3" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="L264" s="3" t="inlineStr"/>
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>school1:11_11</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>Kérjük, jelöld be, mennyire értesz egyet az alábbi állításokkal! - Fontos a jó jegyek megszerzése.</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr"/>
+      <c r="E264" s="2" t="inlineStr"/>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>Please indicate how much you agree with the following statements! - Getting good grades is important.</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr"/>
+      <c r="H264" s="2" t="inlineStr"/>
+      <c r="I264" s="2" t="inlineStr"/>
+      <c r="J264" s="2" t="inlineStr"/>
+      <c r="K264" s="2" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="L264" s="2" t="inlineStr"/>
     </row>
     <row r="265">
-      <c r="A265" s="3" t="inlineStr">
-        <is>
-          <t>some_use1:6_4</t>
-        </is>
-      </c>
-      <c r="B265" s="3" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C265" s="3" t="inlineStr">
-        <is>
-          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Baráti kapcsolatok</t>
-        </is>
-      </c>
-      <c r="D265" s="3" t="inlineStr"/>
-      <c r="E265" s="3" t="inlineStr"/>
-      <c r="F265" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Friendships / relationships with friends | Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="G265" s="3" t="inlineStr">
-        <is>
-          <t>smharm4</t>
-        </is>
-      </c>
-      <c r="H265" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
-        </is>
-      </c>
-      <c r="I265" s="3" t="inlineStr">
-        <is>
-          <t>Relationships with friends</t>
-        </is>
-      </c>
-      <c r="J265" s="3" t="inlineStr">
-        <is>
-          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="K265" s="3" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="L265" s="3" t="inlineStr"/>
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>school_stress1:3_2</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>Iskolai stressz - Kimerültnek érzem magam az iskolai feladatok miatt.</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr"/>
+      <c r="E265" s="2" t="inlineStr"/>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>School stress - I feel exhausted because of school tasks.</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr"/>
+      <c r="H265" s="2" t="inlineStr"/>
+      <c r="I265" s="2" t="inlineStr"/>
+      <c r="J265" s="2" t="inlineStr"/>
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="L265" s="2" t="inlineStr"/>
     </row>
     <row r="266">
-      <c r="A266" s="3" t="inlineStr">
-        <is>
-          <t>some_use1:6_5</t>
-        </is>
-      </c>
-      <c r="B266" s="3" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C266" s="3" t="inlineStr">
-        <is>
-          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Családi kapcsolatok</t>
-        </is>
-      </c>
-      <c r="D266" s="3" t="inlineStr"/>
-      <c r="E266" s="3" t="inlineStr"/>
-      <c r="F266" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Family relationships / relationships with family | Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="G266" s="3" t="inlineStr">
-        <is>
-          <t>smharm5</t>
-        </is>
-      </c>
-      <c r="H266" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
-        </is>
-      </c>
-      <c r="I266" s="3" t="inlineStr">
-        <is>
-          <t>Relationships with family</t>
-        </is>
-      </c>
-      <c r="J266" s="3" t="inlineStr">
-        <is>
-          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="K266" s="3" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="L266" s="3" t="inlineStr"/>
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>school_stress1:3_3</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>Iskolai stressz - Több iskolai feladatom van, mint amennyit kezelni tudok.</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr"/>
+      <c r="E266" s="2" t="inlineStr"/>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>School stress - I have more school tasks than I can handle.</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr"/>
+      <c r="H266" s="2" t="inlineStr"/>
+      <c r="I266" s="2" t="inlineStr"/>
+      <c r="J266" s="2" t="inlineStr"/>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="L266" s="2" t="inlineStr"/>
     </row>
     <row r="267">
-      <c r="A267" s="3" t="inlineStr">
-        <is>
-          <t>some_use1:6_6</t>
-        </is>
-      </c>
-      <c r="B267" s="3" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C267" s="3" t="inlineStr">
-        <is>
-          <t>Kérjük, jelöld meg az alábbi életterületeknél, hogy milyen gyakran van rájuk negatív hatással a telefon, a számítógép vagy a játékkonzol használata! - Szabadtéri tevékenységek vagy sportolás</t>
-        </is>
-      </c>
-      <c r="D267" s="3" t="inlineStr"/>
-      <c r="E267" s="3" t="inlineStr"/>
-      <c r="F267" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect on them! : Outdoor activities or sports | Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="G267" s="3" t="inlineStr">
-        <is>
-          <t>smharm6</t>
-        </is>
-      </c>
-      <c r="H267" s="3" t="inlineStr">
-        <is>
-          <t>For each of the following life areas, please indicate how often your use of phone, computer or gaming console has a negative effect</t>
-        </is>
-      </c>
-      <c r="I267" s="3" t="inlineStr">
-        <is>
-          <t>Doing outdoor activities or sports</t>
-        </is>
-      </c>
-      <c r="J267" s="3" t="inlineStr">
-        <is>
-          <t>Nearly all the time | Often | Sometimes | Rarely | Never</t>
-        </is>
-      </c>
-      <c r="K267" s="3" t="inlineStr">
-        <is>
-          <t>matched</t>
-        </is>
-      </c>
-      <c r="L267" s="3" t="inlineStr"/>
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>schooltype_1_TEXT</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>Melyik felsőoktatási intézménybe, és milyen szakra jársz? - Az alábbi intézménybe és szakra járok: - Text</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr"/>
+      <c r="E267" s="2" t="inlineStr"/>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>Which higher education institution and which program do you attend? - I attend the following institution and program: - Text</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr"/>
+      <c r="H267" s="2" t="inlineStr"/>
+      <c r="I267" s="2" t="inlineStr"/>
+      <c r="J267" s="2" t="inlineStr"/>
+      <c r="K267" s="2" t="inlineStr">
+        <is>
+          <t>extra</t>
+        </is>
+      </c>
+      <c r="L267" s="2" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="5" t="inlineStr">

</xml_diff>